<commit_message>
feat: implement enhanced real-time monitoring with low-price based alerts
- Add multi-level proximity alerts (5%, 3%, 1%)
- Implement buy price reached alerts when low price touches buy lines
- Enhance telegram notifications with current/low price distances
- Remove touch detection alerts as requested
- Update alert logic to use low price for decision making
- Maintain current price and distance calculations for reference
- All systems tested and working correctly
</commit_message>
<xml_diff>
--- a/output/trading_signals.xlsx
+++ b/output/trading_signals.xlsx
@@ -664,7 +664,7 @@
       </c>
       <c r="AH1" s="4" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-16 03:50:19</t>
+          <t>최종 업데이트: 2025-10-16 05:18:52</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       <c r="AD2" s="9" t="inlineStr"/>
       <c r="AE2" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:01</t>
+          <t>2025-10-16 05:18:34</t>
         </is>
       </c>
       <c r="AF2" s="11" t="n">
@@ -827,7 +827,7 @@
       <c r="AD3" s="9" t="inlineStr"/>
       <c r="AE3" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:01</t>
+          <t>2025-10-16 05:18:34</t>
         </is>
       </c>
       <c r="AF3" s="11" t="n">
@@ -911,7 +911,7 @@
       <c r="AD4" s="9" t="inlineStr"/>
       <c r="AE4" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:01</t>
+          <t>2025-10-16 05:18:34</t>
         </is>
       </c>
       <c r="AF4" s="11" t="n">
@@ -995,7 +995,7 @@
       <c r="AD5" s="9" t="inlineStr"/>
       <c r="AE5" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:01</t>
+          <t>2025-10-16 05:18:35</t>
         </is>
       </c>
       <c r="AF5" s="11" t="n">
@@ -1079,7 +1079,7 @@
       <c r="AD6" s="9" t="inlineStr"/>
       <c r="AE6" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:02</t>
+          <t>2025-10-16 05:18:35</t>
         </is>
       </c>
       <c r="AF6" s="11" t="n">
@@ -1163,7 +1163,7 @@
       <c r="AD7" s="9" t="inlineStr"/>
       <c r="AE7" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:02</t>
+          <t>2025-10-16 05:18:35</t>
         </is>
       </c>
       <c r="AF7" s="11" t="n">
@@ -1247,7 +1247,7 @@
       <c r="AD8" s="9" t="inlineStr"/>
       <c r="AE8" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:02</t>
+          <t>2025-10-16 05:18:35</t>
         </is>
       </c>
       <c r="AF8" s="11" t="n">
@@ -1331,7 +1331,7 @@
       <c r="AD9" s="9" t="inlineStr"/>
       <c r="AE9" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:02</t>
+          <t>2025-10-16 05:18:36</t>
         </is>
       </c>
       <c r="AF9" s="11" t="n">
@@ -1415,7 +1415,7 @@
       <c r="AD10" s="9" t="inlineStr"/>
       <c r="AE10" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:03</t>
+          <t>2025-10-16 05:18:36</t>
         </is>
       </c>
       <c r="AF10" s="11" t="n">
@@ -1499,7 +1499,7 @@
       <c r="AD11" s="9" t="inlineStr"/>
       <c r="AE11" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:03</t>
+          <t>2025-10-16 05:18:36</t>
         </is>
       </c>
       <c r="AF11" s="11" t="n">
@@ -1583,7 +1583,7 @@
       <c r="AD12" s="9" t="inlineStr"/>
       <c r="AE12" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:03</t>
+          <t>2025-10-16 05:18:37</t>
         </is>
       </c>
       <c r="AF12" s="11" t="n">
@@ -1667,7 +1667,7 @@
       <c r="AD13" s="9" t="inlineStr"/>
       <c r="AE13" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:04</t>
+          <t>2025-10-16 05:18:37</t>
         </is>
       </c>
       <c r="AF13" s="11" t="n">
@@ -1751,7 +1751,7 @@
       <c r="AD14" s="9" t="inlineStr"/>
       <c r="AE14" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:04</t>
+          <t>2025-10-16 05:18:37</t>
         </is>
       </c>
       <c r="AF14" s="11" t="n">
@@ -1835,7 +1835,7 @@
       <c r="AD15" s="9" t="inlineStr"/>
       <c r="AE15" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:04</t>
+          <t>2025-10-16 05:18:37</t>
         </is>
       </c>
       <c r="AF15" s="11" t="n">
@@ -1919,7 +1919,7 @@
       <c r="AD16" s="9" t="inlineStr"/>
       <c r="AE16" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:04</t>
+          <t>2025-10-16 05:18:38</t>
         </is>
       </c>
       <c r="AF16" s="11" t="n">
@@ -2003,7 +2003,7 @@
       <c r="AD17" s="9" t="inlineStr"/>
       <c r="AE17" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:05</t>
+          <t>2025-10-16 05:18:38</t>
         </is>
       </c>
       <c r="AF17" s="11" t="n">
@@ -2087,7 +2087,7 @@
       <c r="AD18" s="9" t="inlineStr"/>
       <c r="AE18" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:05</t>
+          <t>2025-10-16 05:18:38</t>
         </is>
       </c>
       <c r="AF18" s="11" t="n">
@@ -2171,7 +2171,7 @@
       <c r="AD19" s="9" t="inlineStr"/>
       <c r="AE19" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:05</t>
+          <t>2025-10-16 05:18:38</t>
         </is>
       </c>
       <c r="AF19" s="11" t="n">
@@ -2255,7 +2255,7 @@
       <c r="AD20" s="9" t="inlineStr"/>
       <c r="AE20" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:05</t>
+          <t>2025-10-16 05:18:39</t>
         </is>
       </c>
       <c r="AF20" s="11" t="n">
@@ -2339,7 +2339,7 @@
       <c r="AD21" s="9" t="inlineStr"/>
       <c r="AE21" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:06</t>
+          <t>2025-10-16 05:18:39</t>
         </is>
       </c>
       <c r="AF21" s="11" t="n">
@@ -2423,7 +2423,7 @@
       <c r="AD22" s="9" t="inlineStr"/>
       <c r="AE22" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:06</t>
+          <t>2025-10-16 05:18:39</t>
         </is>
       </c>
       <c r="AF22" s="11" t="n">
@@ -2507,7 +2507,7 @@
       <c r="AD23" s="9" t="inlineStr"/>
       <c r="AE23" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:06</t>
+          <t>2025-10-16 05:18:40</t>
         </is>
       </c>
       <c r="AF23" s="11" t="n">
@@ -2591,7 +2591,7 @@
       <c r="AD24" s="9" t="inlineStr"/>
       <c r="AE24" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:07</t>
+          <t>2025-10-16 05:18:40</t>
         </is>
       </c>
       <c r="AF24" s="11" t="n">
@@ -2675,7 +2675,7 @@
       <c r="AD25" s="9" t="inlineStr"/>
       <c r="AE25" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:07</t>
+          <t>2025-10-16 05:18:40</t>
         </is>
       </c>
       <c r="AF25" s="11" t="n">
@@ -2759,7 +2759,7 @@
       <c r="AD26" s="9" t="inlineStr"/>
       <c r="AE26" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:07</t>
+          <t>2025-10-16 05:18:40</t>
         </is>
       </c>
       <c r="AF26" s="11" t="n">
@@ -2843,7 +2843,7 @@
       <c r="AD27" s="9" t="inlineStr"/>
       <c r="AE27" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:07</t>
+          <t>2025-10-16 05:18:41</t>
         </is>
       </c>
       <c r="AF27" s="11" t="n">
@@ -2927,7 +2927,7 @@
       <c r="AD28" s="9" t="inlineStr"/>
       <c r="AE28" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:08</t>
+          <t>2025-10-16 05:18:41</t>
         </is>
       </c>
       <c r="AF28" s="11" t="n">
@@ -3011,7 +3011,7 @@
       <c r="AD29" s="9" t="inlineStr"/>
       <c r="AE29" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:08</t>
+          <t>2025-10-16 05:18:41</t>
         </is>
       </c>
       <c r="AF29" s="11" t="n">
@@ -3095,7 +3095,7 @@
       <c r="AD30" s="9" t="inlineStr"/>
       <c r="AE30" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:08</t>
+          <t>2025-10-16 05:18:41</t>
         </is>
       </c>
       <c r="AF30" s="11" t="n">
@@ -3179,7 +3179,7 @@
       <c r="AD31" s="9" t="inlineStr"/>
       <c r="AE31" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:08</t>
+          <t>2025-10-16 05:18:42</t>
         </is>
       </c>
       <c r="AF31" s="11" t="n">
@@ -3263,7 +3263,7 @@
       <c r="AD32" s="9" t="inlineStr"/>
       <c r="AE32" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:09</t>
+          <t>2025-10-16 05:18:42</t>
         </is>
       </c>
       <c r="AF32" s="11" t="n">
@@ -3347,7 +3347,7 @@
       <c r="AD33" s="9" t="inlineStr"/>
       <c r="AE33" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:09</t>
+          <t>2025-10-16 05:18:42</t>
         </is>
       </c>
       <c r="AF33" s="11" t="n">
@@ -3431,7 +3431,7 @@
       <c r="AD34" s="9" t="inlineStr"/>
       <c r="AE34" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:09</t>
+          <t>2025-10-16 05:18:43</t>
         </is>
       </c>
       <c r="AF34" s="11" t="n">
@@ -3515,7 +3515,7 @@
       <c r="AD35" s="9" t="inlineStr"/>
       <c r="AE35" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:10</t>
+          <t>2025-10-16 05:18:43</t>
         </is>
       </c>
       <c r="AF35" s="11" t="n">
@@ -3599,7 +3599,7 @@
       <c r="AD36" s="9" t="inlineStr"/>
       <c r="AE36" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:10</t>
+          <t>2025-10-16 05:18:43</t>
         </is>
       </c>
       <c r="AF36" s="11" t="n">
@@ -3683,7 +3683,7 @@
       <c r="AD37" s="9" t="inlineStr"/>
       <c r="AE37" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:10</t>
+          <t>2025-10-16 05:18:43</t>
         </is>
       </c>
       <c r="AF37" s="11" t="n">
@@ -3767,7 +3767,7 @@
       <c r="AD38" s="9" t="inlineStr"/>
       <c r="AE38" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:10</t>
+          <t>2025-10-16 05:18:44</t>
         </is>
       </c>
       <c r="AF38" s="11" t="n">
@@ -3851,7 +3851,7 @@
       <c r="AD39" s="9" t="inlineStr"/>
       <c r="AE39" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:11</t>
+          <t>2025-10-16 05:18:44</t>
         </is>
       </c>
       <c r="AF39" s="11" t="n">
@@ -3935,7 +3935,7 @@
       <c r="AD40" s="9" t="inlineStr"/>
       <c r="AE40" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:11</t>
+          <t>2025-10-16 05:18:44</t>
         </is>
       </c>
       <c r="AF40" s="11" t="n">
@@ -4019,7 +4019,7 @@
       <c r="AD41" s="9" t="inlineStr"/>
       <c r="AE41" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:11</t>
+          <t>2025-10-16 05:18:44</t>
         </is>
       </c>
       <c r="AF41" s="11" t="n">
@@ -4103,7 +4103,7 @@
       <c r="AD42" s="9" t="inlineStr"/>
       <c r="AE42" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:11</t>
+          <t>2025-10-16 05:18:45</t>
         </is>
       </c>
       <c r="AF42" s="11" t="n">
@@ -4187,7 +4187,7 @@
       <c r="AD43" s="9" t="inlineStr"/>
       <c r="AE43" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:12</t>
+          <t>2025-10-16 05:18:45</t>
         </is>
       </c>
       <c r="AF43" s="11" t="n">
@@ -4271,7 +4271,7 @@
       <c r="AD44" s="9" t="inlineStr"/>
       <c r="AE44" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:12</t>
+          <t>2025-10-16 05:18:45</t>
         </is>
       </c>
       <c r="AF44" s="11" t="n">
@@ -4355,7 +4355,7 @@
       <c r="AD45" s="9" t="inlineStr"/>
       <c r="AE45" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:12</t>
+          <t>2025-10-16 05:18:46</t>
         </is>
       </c>
       <c r="AF45" s="11" t="n">
@@ -4439,7 +4439,7 @@
       <c r="AD46" s="9" t="inlineStr"/>
       <c r="AE46" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:13</t>
+          <t>2025-10-16 05:18:46</t>
         </is>
       </c>
       <c r="AF46" s="11" t="n">
@@ -4523,7 +4523,7 @@
       <c r="AD47" s="9" t="inlineStr"/>
       <c r="AE47" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:13</t>
+          <t>2025-10-16 05:18:46</t>
         </is>
       </c>
       <c r="AF47" s="11" t="n">
@@ -4607,7 +4607,7 @@
       <c r="AD48" s="9" t="inlineStr"/>
       <c r="AE48" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:13</t>
+          <t>2025-10-16 05:18:46</t>
         </is>
       </c>
       <c r="AF48" s="11" t="n">
@@ -4691,7 +4691,7 @@
       <c r="AD49" s="9" t="inlineStr"/>
       <c r="AE49" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:13</t>
+          <t>2025-10-16 05:18:47</t>
         </is>
       </c>
       <c r="AF49" s="11" t="n">
@@ -4775,7 +4775,7 @@
       <c r="AD50" s="9" t="inlineStr"/>
       <c r="AE50" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:14</t>
+          <t>2025-10-16 05:18:47</t>
         </is>
       </c>
       <c r="AF50" s="11" t="n">
@@ -4859,7 +4859,7 @@
       <c r="AD51" s="9" t="inlineStr"/>
       <c r="AE51" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:14</t>
+          <t>2025-10-16 05:18:47</t>
         </is>
       </c>
       <c r="AF51" s="11" t="n">
@@ -4943,7 +4943,7 @@
       <c r="AD52" s="9" t="inlineStr"/>
       <c r="AE52" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:14</t>
+          <t>2025-10-16 05:18:47</t>
         </is>
       </c>
       <c r="AF52" s="11" t="n">
@@ -5027,7 +5027,7 @@
       <c r="AD53" s="9" t="inlineStr"/>
       <c r="AE53" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:14</t>
+          <t>2025-10-16 05:18:48</t>
         </is>
       </c>
       <c r="AF53" s="11" t="n">
@@ -5111,7 +5111,7 @@
       <c r="AD54" s="9" t="inlineStr"/>
       <c r="AE54" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:15</t>
+          <t>2025-10-16 05:18:48</t>
         </is>
       </c>
       <c r="AF54" s="11" t="n">
@@ -5195,7 +5195,7 @@
       <c r="AD55" s="9" t="inlineStr"/>
       <c r="AE55" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:15</t>
+          <t>2025-10-16 05:18:48</t>
         </is>
       </c>
       <c r="AF55" s="11" t="n">
@@ -5279,7 +5279,7 @@
       <c r="AD56" s="9" t="inlineStr"/>
       <c r="AE56" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:15</t>
+          <t>2025-10-16 05:18:49</t>
         </is>
       </c>
       <c r="AF56" s="11" t="n">
@@ -5363,7 +5363,7 @@
       <c r="AD57" s="9" t="inlineStr"/>
       <c r="AE57" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:16</t>
+          <t>2025-10-16 05:18:49</t>
         </is>
       </c>
       <c r="AF57" s="11" t="n">
@@ -5447,7 +5447,7 @@
       <c r="AD58" s="9" t="inlineStr"/>
       <c r="AE58" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:16</t>
+          <t>2025-10-16 05:18:49</t>
         </is>
       </c>
       <c r="AF58" s="11" t="n">
@@ -5531,7 +5531,7 @@
       <c r="AD59" s="9" t="inlineStr"/>
       <c r="AE59" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:16</t>
+          <t>2025-10-16 05:18:49</t>
         </is>
       </c>
       <c r="AF59" s="11" t="n">
@@ -5615,7 +5615,7 @@
       <c r="AD60" s="9" t="inlineStr"/>
       <c r="AE60" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:16</t>
+          <t>2025-10-16 05:18:50</t>
         </is>
       </c>
       <c r="AF60" s="11" t="n">
@@ -5699,7 +5699,7 @@
       <c r="AD61" s="9" t="inlineStr"/>
       <c r="AE61" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:17</t>
+          <t>2025-10-16 05:18:50</t>
         </is>
       </c>
       <c r="AF61" s="11" t="n">
@@ -5783,7 +5783,7 @@
       <c r="AD62" s="9" t="inlineStr"/>
       <c r="AE62" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:17</t>
+          <t>2025-10-16 05:18:50</t>
         </is>
       </c>
       <c r="AF62" s="11" t="n">
@@ -5867,7 +5867,7 @@
       <c r="AD63" s="9" t="inlineStr"/>
       <c r="AE63" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:17</t>
+          <t>2025-10-16 05:18:51</t>
         </is>
       </c>
       <c r="AF63" s="11" t="n">
@@ -5951,7 +5951,7 @@
       <c r="AD64" s="9" t="inlineStr"/>
       <c r="AE64" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:18</t>
+          <t>2025-10-16 05:18:51</t>
         </is>
       </c>
       <c r="AF64" s="11" t="n">
@@ -6035,7 +6035,7 @@
       <c r="AD65" s="9" t="inlineStr"/>
       <c r="AE65" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:18</t>
+          <t>2025-10-16 05:18:51</t>
         </is>
       </c>
       <c r="AF65" s="11" t="n">
@@ -6119,7 +6119,7 @@
       <c r="AD66" s="9" t="inlineStr"/>
       <c r="AE66" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:18</t>
+          <t>2025-10-16 05:18:51</t>
         </is>
       </c>
       <c r="AF66" s="11" t="n">
@@ -6203,7 +6203,7 @@
       <c r="AD67" s="9" t="inlineStr"/>
       <c r="AE67" s="10" t="inlineStr">
         <is>
-          <t>2025-10-16 03:50:18</t>
+          <t>2025-10-16 05:18:52</t>
         </is>
       </c>
       <c r="AF67" s="11" t="n">
@@ -6257,7 +6257,7 @@
         <v>34276</v>
       </c>
       <c r="L68" s="8" t="n">
-        <v>1.349048897187536e-13</v>
+        <v>1.349048897187536e-15</v>
       </c>
       <c r="M68" s="9" t="inlineStr"/>
       <c r="N68" s="9" t="inlineStr"/>
@@ -6265,7 +6265,7 @@
         <v>30848.4</v>
       </c>
       <c r="P68" s="8" t="n">
-        <v>2.610054330208374e-13</v>
+        <v>2.610054330208374e-15</v>
       </c>
       <c r="Q68" s="9" t="inlineStr"/>
       <c r="R68" s="9" t="inlineStr"/>
@@ -6273,7 +6273,7 @@
         <v>27763.56</v>
       </c>
       <c r="T68" s="8" t="n">
-        <v>4.011171478009304e-13</v>
+        <v>4.011171478009304e-15</v>
       </c>
       <c r="U68" s="9" t="inlineStr"/>
       <c r="V68" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Add force execution option for testing
- Trading_Signal_System.py: Added --force option
  - Bypasses trading day check when --force is used
  - Normal operation respects trading day restrictions
  - Enhanced logging for force mode

- Real_Time_Monitor.py: Added --force option
  - Bypasses trading day check when --force is used
  - Modified is_monitoring_time() to support force mode
  - Normal operation respects trading day restrictions

- Successfully tested improved tick unit accuracy
  - Verified correct tick units across all price ranges
  - Buy lines now reflect actual Korean stock market standards
  - Force execution confirmed working properly

- Usage: Add --force flag to run on non-trading days for testing
</commit_message>
<xml_diff>
--- a/output/trading_signals.xlsx
+++ b/output/trading_signals.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="AH1" s="3" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-18 10:13:23</t>
+          <t>최종 업데이트: 2025-10-18 10:45:51</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       <c r="AD2" s="8" t="inlineStr"/>
       <c r="AE2" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:03</t>
+          <t>2025-10-18 10:45:27</t>
         </is>
       </c>
       <c r="AF2" s="8" t="inlineStr"/>
@@ -811,7 +811,7 @@
       <c r="AD3" s="8" t="inlineStr"/>
       <c r="AE3" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:03</t>
+          <t>2025-10-18 10:45:27</t>
         </is>
       </c>
       <c r="AF3" s="8" t="inlineStr"/>
@@ -891,7 +891,7 @@
       <c r="AD4" s="8" t="inlineStr"/>
       <c r="AE4" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:03</t>
+          <t>2025-10-18 10:45:27</t>
         </is>
       </c>
       <c r="AF4" s="8" t="inlineStr"/>
@@ -971,7 +971,7 @@
       <c r="AD5" s="8" t="inlineStr"/>
       <c r="AE5" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:04</t>
+          <t>2025-10-18 10:45:28</t>
         </is>
       </c>
       <c r="AF5" s="8" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
       <c r="AD6" s="8" t="inlineStr"/>
       <c r="AE6" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:04</t>
+          <t>2025-10-18 10:45:28</t>
         </is>
       </c>
       <c r="AF6" s="8" t="inlineStr"/>
@@ -1131,7 +1131,7 @@
       <c r="AD7" s="8" t="inlineStr"/>
       <c r="AE7" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:04</t>
+          <t>2025-10-18 10:45:28</t>
         </is>
       </c>
       <c r="AF7" s="8" t="inlineStr"/>
@@ -1211,7 +1211,7 @@
       <c r="AD8" s="8" t="inlineStr"/>
       <c r="AE8" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:04</t>
+          <t>2025-10-18 10:45:29</t>
         </is>
       </c>
       <c r="AF8" s="8" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       <c r="AD9" s="8" t="inlineStr"/>
       <c r="AE9" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:05</t>
+          <t>2025-10-18 10:45:29</t>
         </is>
       </c>
       <c r="AF9" s="8" t="inlineStr"/>
@@ -1371,7 +1371,7 @@
       <c r="AD10" s="8" t="inlineStr"/>
       <c r="AE10" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:05</t>
+          <t>2025-10-18 10:45:29</t>
         </is>
       </c>
       <c r="AF10" s="8" t="inlineStr"/>
@@ -1451,7 +1451,7 @@
       <c r="AD11" s="8" t="inlineStr"/>
       <c r="AE11" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:05</t>
+          <t>2025-10-18 10:45:30</t>
         </is>
       </c>
       <c r="AF11" s="8" t="inlineStr"/>
@@ -1531,7 +1531,7 @@
       <c r="AD12" s="8" t="inlineStr"/>
       <c r="AE12" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:06</t>
+          <t>2025-10-18 10:45:30</t>
         </is>
       </c>
       <c r="AF12" s="8" t="inlineStr"/>
@@ -1611,7 +1611,7 @@
       <c r="AD13" s="8" t="inlineStr"/>
       <c r="AE13" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:06</t>
+          <t>2025-10-18 10:45:31</t>
         </is>
       </c>
       <c r="AF13" s="8" t="inlineStr"/>
@@ -1691,7 +1691,7 @@
       <c r="AD14" s="8" t="inlineStr"/>
       <c r="AE14" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:06</t>
+          <t>2025-10-18 10:45:31</t>
         </is>
       </c>
       <c r="AF14" s="8" t="inlineStr"/>
@@ -1771,7 +1771,7 @@
       <c r="AD15" s="8" t="inlineStr"/>
       <c r="AE15" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:06</t>
+          <t>2025-10-18 10:45:31</t>
         </is>
       </c>
       <c r="AF15" s="8" t="inlineStr"/>
@@ -1851,7 +1851,7 @@
       <c r="AD16" s="8" t="inlineStr"/>
       <c r="AE16" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:07</t>
+          <t>2025-10-18 10:45:31</t>
         </is>
       </c>
       <c r="AF16" s="8" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
       <c r="AD17" s="8" t="inlineStr"/>
       <c r="AE17" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:07</t>
+          <t>2025-10-18 10:45:32</t>
         </is>
       </c>
       <c r="AF17" s="8" t="inlineStr"/>
@@ -2011,7 +2011,7 @@
       <c r="AD18" s="8" t="inlineStr"/>
       <c r="AE18" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:07</t>
+          <t>2025-10-18 10:45:32</t>
         </is>
       </c>
       <c r="AF18" s="8" t="inlineStr"/>
@@ -2091,7 +2091,7 @@
       <c r="AD19" s="8" t="inlineStr"/>
       <c r="AE19" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:07</t>
+          <t>2025-10-18 10:45:32</t>
         </is>
       </c>
       <c r="AF19" s="8" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
       <c r="AD20" s="8" t="inlineStr"/>
       <c r="AE20" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:08</t>
+          <t>2025-10-18 10:45:33</t>
         </is>
       </c>
       <c r="AF20" s="8" t="inlineStr"/>
@@ -2251,7 +2251,7 @@
       <c r="AD21" s="8" t="inlineStr"/>
       <c r="AE21" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:08</t>
+          <t>2025-10-18 10:45:33</t>
         </is>
       </c>
       <c r="AF21" s="8" t="inlineStr"/>
@@ -2331,7 +2331,7 @@
       <c r="AD22" s="8" t="inlineStr"/>
       <c r="AE22" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:08</t>
+          <t>2025-10-18 10:45:33</t>
         </is>
       </c>
       <c r="AF22" s="8" t="inlineStr"/>
@@ -2411,7 +2411,7 @@
       <c r="AD23" s="8" t="inlineStr"/>
       <c r="AE23" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:09</t>
+          <t>2025-10-18 10:45:34</t>
         </is>
       </c>
       <c r="AF23" s="8" t="inlineStr"/>
@@ -2491,7 +2491,7 @@
       <c r="AD24" s="8" t="inlineStr"/>
       <c r="AE24" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:09</t>
+          <t>2025-10-18 10:45:34</t>
         </is>
       </c>
       <c r="AF24" s="8" t="inlineStr"/>
@@ -2571,7 +2571,7 @@
       <c r="AD25" s="8" t="inlineStr"/>
       <c r="AE25" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:09</t>
+          <t>2025-10-18 10:45:34</t>
         </is>
       </c>
       <c r="AF25" s="8" t="inlineStr"/>
@@ -2651,7 +2651,7 @@
       <c r="AD26" s="8" t="inlineStr"/>
       <c r="AE26" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:09</t>
+          <t>2025-10-18 10:45:35</t>
         </is>
       </c>
       <c r="AF26" s="8" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
       <c r="AD27" s="8" t="inlineStr"/>
       <c r="AE27" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:10</t>
+          <t>2025-10-18 10:45:35</t>
         </is>
       </c>
       <c r="AF27" s="8" t="inlineStr"/>
@@ -2811,7 +2811,7 @@
       <c r="AD28" s="8" t="inlineStr"/>
       <c r="AE28" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:10</t>
+          <t>2025-10-18 10:45:35</t>
         </is>
       </c>
       <c r="AF28" s="8" t="inlineStr"/>
@@ -2891,7 +2891,7 @@
       <c r="AD29" s="8" t="inlineStr"/>
       <c r="AE29" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:10</t>
+          <t>2025-10-18 10:45:36</t>
         </is>
       </c>
       <c r="AF29" s="8" t="inlineStr"/>
@@ -2971,7 +2971,7 @@
       <c r="AD30" s="8" t="inlineStr"/>
       <c r="AE30" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:10</t>
+          <t>2025-10-18 10:45:36</t>
         </is>
       </c>
       <c r="AF30" s="8" t="inlineStr"/>
@@ -3051,7 +3051,7 @@
       <c r="AD31" s="8" t="inlineStr"/>
       <c r="AE31" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:11</t>
+          <t>2025-10-18 10:45:36</t>
         </is>
       </c>
       <c r="AF31" s="8" t="inlineStr"/>
@@ -3131,7 +3131,7 @@
       <c r="AD32" s="8" t="inlineStr"/>
       <c r="AE32" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:11</t>
+          <t>2025-10-18 10:45:37</t>
         </is>
       </c>
       <c r="AF32" s="8" t="inlineStr"/>
@@ -3211,7 +3211,7 @@
       <c r="AD33" s="8" t="inlineStr"/>
       <c r="AE33" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:11</t>
+          <t>2025-10-18 10:45:37</t>
         </is>
       </c>
       <c r="AF33" s="8" t="inlineStr"/>
@@ -3291,7 +3291,7 @@
       <c r="AD34" s="8" t="inlineStr"/>
       <c r="AE34" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:12</t>
+          <t>2025-10-18 10:45:38</t>
         </is>
       </c>
       <c r="AF34" s="8" t="inlineStr"/>
@@ -3371,7 +3371,7 @@
       <c r="AD35" s="8" t="inlineStr"/>
       <c r="AE35" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:12</t>
+          <t>2025-10-18 10:45:38</t>
         </is>
       </c>
       <c r="AF35" s="8" t="inlineStr"/>
@@ -3451,7 +3451,7 @@
       <c r="AD36" s="8" t="inlineStr"/>
       <c r="AE36" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:12</t>
+          <t>2025-10-18 10:45:38</t>
         </is>
       </c>
       <c r="AF36" s="8" t="inlineStr"/>
@@ -3531,7 +3531,7 @@
       <c r="AD37" s="8" t="inlineStr"/>
       <c r="AE37" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:12</t>
+          <t>2025-10-18 10:45:39</t>
         </is>
       </c>
       <c r="AF37" s="8" t="inlineStr"/>
@@ -3611,7 +3611,7 @@
       <c r="AD38" s="8" t="inlineStr"/>
       <c r="AE38" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:13</t>
+          <t>2025-10-18 10:45:39</t>
         </is>
       </c>
       <c r="AF38" s="8" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       <c r="AD39" s="8" t="inlineStr"/>
       <c r="AE39" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:13</t>
+          <t>2025-10-18 10:45:39</t>
         </is>
       </c>
       <c r="AF39" s="8" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
       <c r="AD40" s="8" t="inlineStr"/>
       <c r="AE40" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:13</t>
+          <t>2025-10-18 10:45:40</t>
         </is>
       </c>
       <c r="AF40" s="8" t="inlineStr"/>
@@ -3851,7 +3851,7 @@
       <c r="AD41" s="8" t="inlineStr"/>
       <c r="AE41" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:14</t>
+          <t>2025-10-18 10:45:40</t>
         </is>
       </c>
       <c r="AF41" s="8" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       <c r="AD42" s="8" t="inlineStr"/>
       <c r="AE42" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:14</t>
+          <t>2025-10-18 10:45:40</t>
         </is>
       </c>
       <c r="AF42" s="8" t="inlineStr"/>
@@ -4011,7 +4011,7 @@
       <c r="AD43" s="8" t="inlineStr"/>
       <c r="AE43" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:14</t>
+          <t>2025-10-18 10:45:41</t>
         </is>
       </c>
       <c r="AF43" s="8" t="inlineStr"/>
@@ -4091,7 +4091,7 @@
       <c r="AD44" s="8" t="inlineStr"/>
       <c r="AE44" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:14</t>
+          <t>2025-10-18 10:45:41</t>
         </is>
       </c>
       <c r="AF44" s="8" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       <c r="AD45" s="8" t="inlineStr"/>
       <c r="AE45" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:15</t>
+          <t>2025-10-18 10:45:41</t>
         </is>
       </c>
       <c r="AF45" s="8" t="inlineStr"/>
@@ -4251,7 +4251,7 @@
       <c r="AD46" s="8" t="inlineStr"/>
       <c r="AE46" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:15</t>
+          <t>2025-10-18 10:45:42</t>
         </is>
       </c>
       <c r="AF46" s="8" t="inlineStr"/>
@@ -4331,7 +4331,7 @@
       <c r="AD47" s="8" t="inlineStr"/>
       <c r="AE47" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:15</t>
+          <t>2025-10-18 10:45:42</t>
         </is>
       </c>
       <c r="AF47" s="8" t="inlineStr"/>
@@ -4411,7 +4411,7 @@
       <c r="AD48" s="8" t="inlineStr"/>
       <c r="AE48" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:15</t>
+          <t>2025-10-18 10:45:42</t>
         </is>
       </c>
       <c r="AF48" s="8" t="inlineStr"/>
@@ -4491,7 +4491,7 @@
       <c r="AD49" s="8" t="inlineStr"/>
       <c r="AE49" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:16</t>
+          <t>2025-10-18 10:45:43</t>
         </is>
       </c>
       <c r="AF49" s="8" t="inlineStr"/>
@@ -4571,7 +4571,7 @@
       <c r="AD50" s="8" t="inlineStr"/>
       <c r="AE50" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:16</t>
+          <t>2025-10-18 10:45:43</t>
         </is>
       </c>
       <c r="AF50" s="8" t="inlineStr"/>
@@ -4651,7 +4651,7 @@
       <c r="AD51" s="8" t="inlineStr"/>
       <c r="AE51" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:16</t>
+          <t>2025-10-18 10:45:43</t>
         </is>
       </c>
       <c r="AF51" s="8" t="inlineStr"/>
@@ -4731,7 +4731,7 @@
       <c r="AD52" s="8" t="inlineStr"/>
       <c r="AE52" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:17</t>
+          <t>2025-10-18 10:45:44</t>
         </is>
       </c>
       <c r="AF52" s="8" t="inlineStr"/>
@@ -4811,7 +4811,7 @@
       <c r="AD53" s="8" t="inlineStr"/>
       <c r="AE53" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:17</t>
+          <t>2025-10-18 10:45:44</t>
         </is>
       </c>
       <c r="AF53" s="8" t="inlineStr"/>
@@ -4891,7 +4891,7 @@
       <c r="AD54" s="8" t="inlineStr"/>
       <c r="AE54" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:17</t>
+          <t>2025-10-18 10:45:44</t>
         </is>
       </c>
       <c r="AF54" s="8" t="inlineStr"/>
@@ -4971,7 +4971,7 @@
       <c r="AD55" s="8" t="inlineStr"/>
       <c r="AE55" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:17</t>
+          <t>2025-10-18 10:45:44</t>
         </is>
       </c>
       <c r="AF55" s="8" t="inlineStr"/>
@@ -5051,7 +5051,7 @@
       <c r="AD56" s="8" t="inlineStr"/>
       <c r="AE56" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:18</t>
+          <t>2025-10-18 10:45:45</t>
         </is>
       </c>
       <c r="AF56" s="8" t="inlineStr"/>
@@ -5131,7 +5131,7 @@
       <c r="AD57" s="8" t="inlineStr"/>
       <c r="AE57" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:18</t>
+          <t>2025-10-18 10:45:45</t>
         </is>
       </c>
       <c r="AF57" s="8" t="inlineStr"/>
@@ -5211,7 +5211,7 @@
       <c r="AD58" s="8" t="inlineStr"/>
       <c r="AE58" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:18</t>
+          <t>2025-10-18 10:45:45</t>
         </is>
       </c>
       <c r="AF58" s="8" t="inlineStr"/>
@@ -5291,7 +5291,7 @@
       <c r="AD59" s="8" t="inlineStr"/>
       <c r="AE59" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:19</t>
+          <t>2025-10-18 10:45:46</t>
         </is>
       </c>
       <c r="AF59" s="8" t="inlineStr"/>
@@ -5371,7 +5371,7 @@
       <c r="AD60" s="8" t="inlineStr"/>
       <c r="AE60" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:19</t>
+          <t>2025-10-18 10:45:46</t>
         </is>
       </c>
       <c r="AF60" s="8" t="inlineStr"/>
@@ -5451,7 +5451,7 @@
       <c r="AD61" s="8" t="inlineStr"/>
       <c r="AE61" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:19</t>
+          <t>2025-10-18 10:45:46</t>
         </is>
       </c>
       <c r="AF61" s="8" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
       <c r="AD62" s="8" t="inlineStr"/>
       <c r="AE62" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:19</t>
+          <t>2025-10-18 10:45:47</t>
         </is>
       </c>
       <c r="AF62" s="8" t="inlineStr"/>
@@ -5611,7 +5611,7 @@
       <c r="AD63" s="8" t="inlineStr"/>
       <c r="AE63" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:20</t>
+          <t>2025-10-18 10:45:47</t>
         </is>
       </c>
       <c r="AF63" s="8" t="inlineStr"/>
@@ -5691,7 +5691,7 @@
       <c r="AD64" s="8" t="inlineStr"/>
       <c r="AE64" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:20</t>
+          <t>2025-10-18 10:45:47</t>
         </is>
       </c>
       <c r="AF64" s="8" t="inlineStr"/>
@@ -5771,7 +5771,7 @@
       <c r="AD65" s="8" t="inlineStr"/>
       <c r="AE65" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:20</t>
+          <t>2025-10-18 10:45:48</t>
         </is>
       </c>
       <c r="AF65" s="8" t="inlineStr"/>
@@ -5851,7 +5851,7 @@
       <c r="AD66" s="8" t="inlineStr"/>
       <c r="AE66" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:21</t>
+          <t>2025-10-18 10:45:48</t>
         </is>
       </c>
       <c r="AF66" s="8" t="inlineStr"/>
@@ -5931,7 +5931,7 @@
       <c r="AD67" s="8" t="inlineStr"/>
       <c r="AE67" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:21</t>
+          <t>2025-10-18 10:45:49</t>
         </is>
       </c>
       <c r="AF67" s="8" t="inlineStr"/>
@@ -6011,7 +6011,7 @@
       <c r="AD68" s="8" t="inlineStr"/>
       <c r="AE68" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:21</t>
+          <t>2025-10-18 10:45:49</t>
         </is>
       </c>
       <c r="AF68" s="8" t="inlineStr"/>
@@ -6091,7 +6091,7 @@
       <c r="AD69" s="8" t="inlineStr"/>
       <c r="AE69" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:21</t>
+          <t>2025-10-18 10:45:49</t>
         </is>
       </c>
       <c r="AF69" s="8" t="inlineStr"/>
@@ -6171,7 +6171,7 @@
       <c r="AD70" s="8" t="inlineStr"/>
       <c r="AE70" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:22</t>
+          <t>2025-10-18 10:45:50</t>
         </is>
       </c>
       <c r="AF70" s="8" t="inlineStr"/>
@@ -6251,7 +6251,7 @@
       <c r="AD71" s="8" t="inlineStr"/>
       <c r="AE71" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:22</t>
+          <t>2025-10-18 10:45:50</t>
         </is>
       </c>
       <c r="AF71" s="8" t="inlineStr"/>
@@ -6331,7 +6331,7 @@
       <c r="AD72" s="8" t="inlineStr"/>
       <c r="AE72" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:22</t>
+          <t>2025-10-18 10:45:50</t>
         </is>
       </c>
       <c r="AF72" s="8" t="inlineStr"/>
@@ -6411,7 +6411,7 @@
       <c r="AD73" s="8" t="inlineStr"/>
       <c r="AE73" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:13:22</t>
+          <t>2025-10-18 10:45:51</t>
         </is>
       </c>
       <c r="AF73" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix Korean stock market tick unit to exact standards
- Trading_Signal_System.py: Updated get_tick_unit function
  - Applied exact Korean stock market tick unit standards
  - 2,000??誘몃쭔: 1?? 2,000~5,000?? 5?? 5,000~20,000?? 10??  - 20,000~50,000?? 50?? 50,000~200,000?? 100??  - 200,000~500,000?? 500?? 500,000???댁긽: 1,000??
- Real_Time_Monitor.py: Updated calculate_tick_unit function
  - Applied exact Korean stock market tick unit standards
  - Consistent with Trading_Signal_System.py

- Key improvements:
  - Samsung SDI: 171,580????169,460??(100??tick instead of 500??
  - NAVER: 200,740????199,780??(100??tick instead of 500??
  - More accurate buy lines reflecting actual purchasable prices

- Tested successfully with force execution mode
- All buy lines now use correct Korean stock market tick units
</commit_message>
<xml_diff>
--- a/output/trading_signals.xlsx
+++ b/output/trading_signals.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="AH1" s="3" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-18 10:45:51</t>
+          <t>최종 업데이트: 2025-10-18 11:06:03</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       <c r="AD2" s="8" t="inlineStr"/>
       <c r="AE2" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:27</t>
+          <t>2025-10-18 11:05:39</t>
         </is>
       </c>
       <c r="AF2" s="8" t="inlineStr"/>
@@ -811,7 +811,7 @@
       <c r="AD3" s="8" t="inlineStr"/>
       <c r="AE3" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:27</t>
+          <t>2025-10-18 11:05:39</t>
         </is>
       </c>
       <c r="AF3" s="8" t="inlineStr"/>
@@ -891,7 +891,7 @@
       <c r="AD4" s="8" t="inlineStr"/>
       <c r="AE4" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:27</t>
+          <t>2025-10-18 11:05:39</t>
         </is>
       </c>
       <c r="AF4" s="8" t="inlineStr"/>
@@ -919,7 +919,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 25.1%</t>
+          <t>1차 매수선까지 25.4%</t>
         </is>
       </c>
       <c r="F5" s="6" t="n">
@@ -938,26 +938,26 @@
         <v>199680</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>200180</v>
+        <v>199780</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>25.13737636127485</v>
+        <v>25.38792671939133</v>
       </c>
       <c r="M5" s="8" t="inlineStr"/>
       <c r="N5" s="8" t="inlineStr"/>
       <c r="O5" s="6" t="n">
-        <v>180662</v>
+        <v>179902</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>38.65671807020846</v>
+        <v>39.24247645940568</v>
       </c>
       <c r="Q5" s="8" t="inlineStr"/>
       <c r="R5" s="8" t="inlineStr"/>
       <c r="S5" s="6" t="n">
-        <v>163095.8</v>
+        <v>162011.8</v>
       </c>
       <c r="T5" s="7" t="n">
-        <v>53.59071171667203</v>
+        <v>54.61836730410992</v>
       </c>
       <c r="U5" s="8" t="inlineStr"/>
       <c r="V5" s="8" t="inlineStr"/>
@@ -971,7 +971,7 @@
       <c r="AD5" s="8" t="inlineStr"/>
       <c r="AE5" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:28</t>
+          <t>2025-10-18 11:05:40</t>
         </is>
       </c>
       <c r="AF5" s="8" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
       <c r="AD6" s="8" t="inlineStr"/>
       <c r="AE6" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:28</t>
+          <t>2025-10-18 11:05:40</t>
         </is>
       </c>
       <c r="AF6" s="8" t="inlineStr"/>
@@ -1131,7 +1131,7 @@
       <c r="AD7" s="8" t="inlineStr"/>
       <c r="AE7" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:28</t>
+          <t>2025-10-18 11:05:40</t>
         </is>
       </c>
       <c r="AF7" s="8" t="inlineStr"/>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 46.6%</t>
+          <t>1차 매수선까지 46.9%</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
@@ -1178,26 +1178,26 @@
         <v>169360</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>169860</v>
+        <v>169460</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>46.59131049099258</v>
+        <v>46.93733034344388</v>
       </c>
       <c r="M8" s="8" t="inlineStr"/>
       <c r="N8" s="8" t="inlineStr"/>
       <c r="O8" s="6" t="n">
-        <v>153374</v>
+        <v>152614</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>62.34824676933509</v>
+        <v>63.15672218800372</v>
       </c>
       <c r="Q8" s="8" t="inlineStr"/>
       <c r="R8" s="8" t="inlineStr"/>
       <c r="S8" s="6" t="n">
-        <v>138536.6</v>
+        <v>137452.6</v>
       </c>
       <c r="T8" s="7" t="n">
-        <v>79.73589650677148</v>
+        <v>81.15335759381779</v>
       </c>
       <c r="U8" s="8" t="inlineStr"/>
       <c r="V8" s="8" t="inlineStr"/>
@@ -1211,7 +1211,7 @@
       <c r="AD8" s="8" t="inlineStr"/>
       <c r="AE8" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:29</t>
+          <t>2025-10-18 11:05:41</t>
         </is>
       </c>
       <c r="AF8" s="8" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       <c r="AD9" s="8" t="inlineStr"/>
       <c r="AE9" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:29</t>
+          <t>2025-10-18 11:05:41</t>
         </is>
       </c>
       <c r="AF9" s="8" t="inlineStr"/>
@@ -1371,7 +1371,7 @@
       <c r="AD10" s="8" t="inlineStr"/>
       <c r="AE10" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:29</t>
+          <t>2025-10-18 11:05:41</t>
         </is>
       </c>
       <c r="AF10" s="8" t="inlineStr"/>
@@ -1451,7 +1451,7 @@
       <c r="AD11" s="8" t="inlineStr"/>
       <c r="AE11" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:30</t>
+          <t>2025-10-18 11:05:42</t>
         </is>
       </c>
       <c r="AF11" s="8" t="inlineStr"/>
@@ -1531,7 +1531,7 @@
       <c r="AD12" s="8" t="inlineStr"/>
       <c r="AE12" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:30</t>
+          <t>2025-10-18 11:05:42</t>
         </is>
       </c>
       <c r="AF12" s="8" t="inlineStr"/>
@@ -1611,7 +1611,7 @@
       <c r="AD13" s="8" t="inlineStr"/>
       <c r="AE13" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:31</t>
+          <t>2025-10-18 11:05:42</t>
         </is>
       </c>
       <c r="AF13" s="8" t="inlineStr"/>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 36.3%</t>
+          <t>1차 매수선까지 36.6%</t>
         </is>
       </c>
       <c r="F14" s="6" t="n">
@@ -1658,26 +1658,26 @@
         <v>175960</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>176460</v>
+        <v>176060</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>36.29151082398277</v>
+        <v>36.60115869589913</v>
       </c>
       <c r="M14" s="8" t="inlineStr"/>
       <c r="N14" s="8" t="inlineStr"/>
       <c r="O14" s="6" t="n">
-        <v>159314</v>
+        <v>158554</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>50.9597398847559</v>
+        <v>51.68333816869962</v>
       </c>
       <c r="Q14" s="8" t="inlineStr"/>
       <c r="R14" s="8" t="inlineStr"/>
       <c r="S14" s="6" t="n">
-        <v>143882.6</v>
+        <v>142798.6</v>
       </c>
       <c r="T14" s="7" t="n">
-        <v>67.15016270209185</v>
+        <v>68.41901811362295</v>
       </c>
       <c r="U14" s="8" t="inlineStr"/>
       <c r="V14" s="8" t="inlineStr"/>
@@ -1691,7 +1691,7 @@
       <c r="AD14" s="8" t="inlineStr"/>
       <c r="AE14" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:31</t>
+          <t>2025-10-18 11:05:43</t>
         </is>
       </c>
       <c r="AF14" s="8" t="inlineStr"/>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 53.9%</t>
+          <t>1차 매수선까지 54.4%</t>
         </is>
       </c>
       <c r="F15" s="6" t="n">
@@ -1738,26 +1738,26 @@
         <v>119952</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>120452</v>
+        <v>120052</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>53.92023378607246</v>
+        <v>54.4330789991004</v>
       </c>
       <c r="M15" s="8" t="inlineStr"/>
       <c r="N15" s="8" t="inlineStr"/>
       <c r="O15" s="6" t="n">
-        <v>108906.8</v>
+        <v>108146.8</v>
       </c>
       <c r="P15" s="7" t="n">
-        <v>70.23730382308541</v>
+        <v>71.4336438988486</v>
       </c>
       <c r="Q15" s="8" t="inlineStr"/>
       <c r="R15" s="8" t="inlineStr"/>
       <c r="S15" s="6" t="n">
-        <v>98116.12000000001</v>
+        <v>97432.12000000001</v>
       </c>
       <c r="T15" s="7" t="n">
-        <v>88.95977541712817</v>
+        <v>90.2863244687686</v>
       </c>
       <c r="U15" s="8" t="inlineStr"/>
       <c r="V15" s="8" t="inlineStr"/>
@@ -1771,7 +1771,7 @@
       <c r="AD15" s="8" t="inlineStr"/>
       <c r="AE15" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:31</t>
+          <t>2025-10-18 11:05:43</t>
         </is>
       </c>
       <c r="AF15" s="8" t="inlineStr"/>
@@ -1851,7 +1851,7 @@
       <c r="AD16" s="8" t="inlineStr"/>
       <c r="AE16" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:31</t>
+          <t>2025-10-18 11:05:43</t>
         </is>
       </c>
       <c r="AF16" s="8" t="inlineStr"/>
@@ -1914,10 +1914,10 @@
       <c r="Q17" s="8" t="inlineStr"/>
       <c r="R17" s="8" t="inlineStr"/>
       <c r="S17" s="6" t="n">
-        <v>190749.2</v>
+        <v>190349.2</v>
       </c>
       <c r="T17" s="7" t="n">
-        <v>73.78840907327526</v>
+        <v>74.15360821059399</v>
       </c>
       <c r="U17" s="8" t="inlineStr"/>
       <c r="V17" s="8" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
       <c r="AD17" s="8" t="inlineStr"/>
       <c r="AE17" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:32</t>
+          <t>2025-10-18 11:05:44</t>
         </is>
       </c>
       <c r="AF17" s="8" t="inlineStr"/>
@@ -2011,7 +2011,7 @@
       <c r="AD18" s="8" t="inlineStr"/>
       <c r="AE18" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:32</t>
+          <t>2025-10-18 11:05:44</t>
         </is>
       </c>
       <c r="AF18" s="8" t="inlineStr"/>
@@ -2091,7 +2091,7 @@
       <c r="AD19" s="8" t="inlineStr"/>
       <c r="AE19" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:32</t>
+          <t>2025-10-18 11:05:44</t>
         </is>
       </c>
       <c r="AF19" s="8" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
       <c r="AD20" s="8" t="inlineStr"/>
       <c r="AE20" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:33</t>
+          <t>2025-10-18 11:05:45</t>
         </is>
       </c>
       <c r="AF20" s="8" t="inlineStr"/>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 55.9%</t>
+          <t>1차 매수선까지 56.4%</t>
         </is>
       </c>
       <c r="F21" s="6" t="n">
@@ -2218,26 +2218,26 @@
         <v>122759.52</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>123259.52</v>
+        <v>122859.52</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>55.93116053023734</v>
+        <v>56.43883355559259</v>
       </c>
       <c r="M21" s="8" t="inlineStr"/>
       <c r="N21" s="8" t="inlineStr"/>
       <c r="O21" s="6" t="n">
-        <v>111433.568</v>
+        <v>110673.568</v>
       </c>
       <c r="P21" s="7" t="n">
-        <v>72.47944533194881</v>
+        <v>73.66386886523799</v>
       </c>
       <c r="Q21" s="8" t="inlineStr"/>
       <c r="R21" s="8" t="inlineStr"/>
       <c r="S21" s="6" t="n">
-        <v>100790.2112</v>
+        <v>99706.21120000001</v>
       </c>
       <c r="T21" s="7" t="n">
-        <v>90.69312159552256</v>
+        <v>92.76632587559399</v>
       </c>
       <c r="U21" s="8" t="inlineStr"/>
       <c r="V21" s="8" t="inlineStr"/>
@@ -2251,7 +2251,7 @@
       <c r="AD21" s="8" t="inlineStr"/>
       <c r="AE21" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:33</t>
+          <t>2025-10-18 11:05:45</t>
         </is>
       </c>
       <c r="AF21" s="8" t="inlineStr"/>
@@ -2331,7 +2331,7 @@
       <c r="AD22" s="8" t="inlineStr"/>
       <c r="AE22" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:33</t>
+          <t>2025-10-18 11:05:45</t>
         </is>
       </c>
       <c r="AF22" s="8" t="inlineStr"/>
@@ -2386,18 +2386,18 @@
       <c r="M23" s="8" t="inlineStr"/>
       <c r="N23" s="8" t="inlineStr"/>
       <c r="O23" s="6" t="n">
-        <v>19252.4</v>
+        <v>19212.4</v>
       </c>
       <c r="P23" s="7" t="n">
-        <v>13.75205169225654</v>
+        <v>13.98888218025857</v>
       </c>
       <c r="Q23" s="8" t="inlineStr"/>
       <c r="R23" s="8" t="inlineStr"/>
       <c r="S23" s="6" t="n">
-        <v>17377.16</v>
+        <v>17301.16</v>
       </c>
       <c r="T23" s="7" t="n">
-        <v>26.02749816425696</v>
+        <v>26.5811078563518</v>
       </c>
       <c r="U23" s="8" t="inlineStr"/>
       <c r="V23" s="8" t="inlineStr"/>
@@ -2411,7 +2411,7 @@
       <c r="AD23" s="8" t="inlineStr"/>
       <c r="AE23" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:34</t>
+          <t>2025-10-18 11:05:46</t>
         </is>
       </c>
       <c r="AF23" s="8" t="inlineStr"/>
@@ -2491,7 +2491,7 @@
       <c r="AD24" s="8" t="inlineStr"/>
       <c r="AE24" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:34</t>
+          <t>2025-10-18 11:05:46</t>
         </is>
       </c>
       <c r="AF24" s="8" t="inlineStr"/>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 18.8%</t>
+          <t>1차 매수선까지 19.2%</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
@@ -2538,26 +2538,26 @@
         <v>13321.2</v>
       </c>
       <c r="K25" s="6" t="n">
-        <v>13371.2</v>
+        <v>13331.2</v>
       </c>
       <c r="L25" s="7" t="n">
-        <v>18.83750149575206</v>
+        <v>19.19407105136821</v>
       </c>
       <c r="M25" s="8" t="inlineStr"/>
       <c r="N25" s="8" t="inlineStr"/>
       <c r="O25" s="6" t="n">
-        <v>12084.08</v>
+        <v>12008.08</v>
       </c>
       <c r="P25" s="7" t="n">
-        <v>31.49532277177905</v>
+        <v>32.32756610548896</v>
       </c>
       <c r="Q25" s="8" t="inlineStr"/>
       <c r="R25" s="8" t="inlineStr"/>
       <c r="S25" s="6" t="n">
-        <v>10925.672</v>
+        <v>10817.272</v>
       </c>
       <c r="T25" s="7" t="n">
-        <v>45.43727836603549</v>
+        <v>46.89470690946845</v>
       </c>
       <c r="U25" s="8" t="inlineStr"/>
       <c r="V25" s="8" t="inlineStr"/>
@@ -2571,7 +2571,7 @@
       <c r="AD25" s="8" t="inlineStr"/>
       <c r="AE25" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:34</t>
+          <t>2025-10-18 11:05:46</t>
         </is>
       </c>
       <c r="AF25" s="8" t="inlineStr"/>
@@ -2651,7 +2651,7 @@
       <c r="AD26" s="8" t="inlineStr"/>
       <c r="AE26" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:35</t>
+          <t>2025-10-18 11:05:47</t>
         </is>
       </c>
       <c r="AF26" s="8" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
       <c r="AD27" s="8" t="inlineStr"/>
       <c r="AE27" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:35</t>
+          <t>2025-10-18 11:05:47</t>
         </is>
       </c>
       <c r="AF27" s="8" t="inlineStr"/>
@@ -2811,7 +2811,7 @@
       <c r="AD28" s="8" t="inlineStr"/>
       <c r="AE28" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:35</t>
+          <t>2025-10-18 11:05:48</t>
         </is>
       </c>
       <c r="AF28" s="8" t="inlineStr"/>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 24.7%</t>
+          <t>1차 매수선까지 25.1%</t>
         </is>
       </c>
       <c r="F29" s="6" t="n">
@@ -2858,26 +2858,26 @@
         <v>138716</v>
       </c>
       <c r="K29" s="6" t="n">
-        <v>139216</v>
+        <v>138816</v>
       </c>
       <c r="L29" s="7" t="n">
-        <v>24.6983105390185</v>
+        <v>25.05763024435224</v>
       </c>
       <c r="M29" s="8" t="inlineStr"/>
       <c r="N29" s="8" t="inlineStr"/>
       <c r="O29" s="6" t="n">
-        <v>125794.4</v>
+        <v>125034.4</v>
       </c>
       <c r="P29" s="7" t="n">
-        <v>38.00296356594569</v>
+        <v>38.84179073918857</v>
       </c>
       <c r="Q29" s="8" t="inlineStr"/>
       <c r="R29" s="8" t="inlineStr"/>
       <c r="S29" s="6" t="n">
-        <v>113714.96</v>
+        <v>112630.96</v>
       </c>
       <c r="T29" s="7" t="n">
-        <v>52.66241134851561</v>
+        <v>54.13168812553848</v>
       </c>
       <c r="U29" s="8" t="inlineStr"/>
       <c r="V29" s="8" t="inlineStr"/>
@@ -2891,7 +2891,7 @@
       <c r="AD29" s="8" t="inlineStr"/>
       <c r="AE29" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:36</t>
+          <t>2025-10-18 11:05:48</t>
         </is>
       </c>
       <c r="AF29" s="8" t="inlineStr"/>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 8.6% (접근 중!)</t>
+          <t>1차 매수선까지 8.9% (접근 중!)</t>
         </is>
       </c>
       <c r="F30" s="6" t="n">
@@ -2938,26 +2938,26 @@
         <v>147728</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>148228</v>
+        <v>147828</v>
       </c>
       <c r="L30" s="7" t="n">
-        <v>8.616455730361334</v>
+        <v>8.91035527775523</v>
       </c>
       <c r="M30" s="8" t="inlineStr"/>
       <c r="N30" s="8" t="inlineStr"/>
       <c r="O30" s="6" t="n">
-        <v>133905.2</v>
+        <v>133145.2</v>
       </c>
       <c r="P30" s="7" t="n">
-        <v>20.23431502286691</v>
+        <v>20.92061899339967</v>
       </c>
       <c r="Q30" s="8" t="inlineStr"/>
       <c r="R30" s="8" t="inlineStr"/>
       <c r="S30" s="6" t="n">
-        <v>121014.68</v>
+        <v>119930.68</v>
       </c>
       <c r="T30" s="7" t="n">
-        <v>33.04171031150931</v>
+        <v>34.24421507490826</v>
       </c>
       <c r="U30" s="8" t="inlineStr"/>
       <c r="V30" s="8" t="inlineStr"/>
@@ -2971,7 +2971,7 @@
       <c r="AD30" s="8" t="inlineStr"/>
       <c r="AE30" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:36</t>
+          <t>2025-10-18 11:05:48</t>
         </is>
       </c>
       <c r="AF30" s="8" t="inlineStr"/>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 13.6%</t>
+          <t>1차 매수선까지 13.9%</t>
         </is>
       </c>
       <c r="F31" s="6" t="n">
@@ -3018,26 +3018,26 @@
         <v>175040</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>175540</v>
+        <v>175140</v>
       </c>
       <c r="L31" s="7" t="n">
-        <v>13.64931069841631</v>
+        <v>13.90887290167866</v>
       </c>
       <c r="M31" s="8" t="inlineStr"/>
       <c r="N31" s="8" t="inlineStr"/>
       <c r="O31" s="6" t="n">
-        <v>158486</v>
+        <v>157726</v>
       </c>
       <c r="P31" s="7" t="n">
-        <v>25.87862650328735</v>
+        <v>26.48517048552553</v>
       </c>
       <c r="Q31" s="8" t="inlineStr"/>
       <c r="R31" s="8" t="inlineStr"/>
       <c r="S31" s="6" t="n">
-        <v>143137.4</v>
+        <v>142053.4</v>
       </c>
       <c r="T31" s="7" t="n">
-        <v>39.37657104292798</v>
+        <v>40.4401443400862</v>
       </c>
       <c r="U31" s="8" t="inlineStr"/>
       <c r="V31" s="8" t="inlineStr"/>
@@ -3051,7 +3051,7 @@
       <c r="AD31" s="8" t="inlineStr"/>
       <c r="AE31" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:36</t>
+          <t>2025-10-18 11:05:49</t>
         </is>
       </c>
       <c r="AF31" s="8" t="inlineStr"/>
@@ -3131,7 +3131,7 @@
       <c r="AD32" s="8" t="inlineStr"/>
       <c r="AE32" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:37</t>
+          <t>2025-10-18 11:05:49</t>
         </is>
       </c>
       <c r="AF32" s="8" t="inlineStr"/>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 15.6%</t>
+          <t>1차 매수선까지 15.9%</t>
         </is>
       </c>
       <c r="F33" s="6" t="n">
@@ -3178,26 +3178,26 @@
         <v>173380</v>
       </c>
       <c r="K33" s="6" t="n">
-        <v>173880</v>
+        <v>173480</v>
       </c>
       <c r="L33" s="7" t="n">
-        <v>15.59696342305038</v>
+        <v>15.86350011528707</v>
       </c>
       <c r="M33" s="8" t="inlineStr"/>
       <c r="N33" s="8" t="inlineStr"/>
       <c r="O33" s="6" t="n">
-        <v>156992</v>
+        <v>156232</v>
       </c>
       <c r="P33" s="7" t="n">
-        <v>28.03200163065634</v>
+        <v>28.65482103538328</v>
       </c>
       <c r="Q33" s="8" t="inlineStr"/>
       <c r="R33" s="8" t="inlineStr"/>
       <c r="S33" s="6" t="n">
-        <v>141792.8</v>
+        <v>140708.8</v>
       </c>
       <c r="T33" s="7" t="n">
-        <v>41.75613994504656</v>
+        <v>42.84820849868663</v>
       </c>
       <c r="U33" s="8" t="inlineStr"/>
       <c r="V33" s="8" t="inlineStr"/>
@@ -3211,7 +3211,7 @@
       <c r="AD33" s="8" t="inlineStr"/>
       <c r="AE33" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:37</t>
+          <t>2025-10-18 11:05:49</t>
         </is>
       </c>
       <c r="AF33" s="8" t="inlineStr"/>
@@ -3291,7 +3291,7 @@
       <c r="AD34" s="8" t="inlineStr"/>
       <c r="AE34" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:38</t>
+          <t>2025-10-18 11:05:50</t>
         </is>
       </c>
       <c r="AF34" s="8" t="inlineStr"/>
@@ -3371,7 +3371,7 @@
       <c r="AD35" s="8" t="inlineStr"/>
       <c r="AE35" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:38</t>
+          <t>2025-10-18 11:05:50</t>
         </is>
       </c>
       <c r="AF35" s="8" t="inlineStr"/>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 0.9% (접근 중!)</t>
+          <t>1차 매수선까지 1.1% (접근 중!)</t>
         </is>
       </c>
       <c r="F36" s="6" t="n">
@@ -3418,26 +3418,26 @@
         <v>164336</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>164836</v>
+        <v>164436</v>
       </c>
       <c r="L36" s="7" t="n">
-        <v>0.8881555000121333</v>
+        <v>1.133571723953392</v>
       </c>
       <c r="M36" s="8" t="inlineStr"/>
       <c r="N36" s="8" t="inlineStr"/>
       <c r="O36" s="6" t="n">
-        <v>148852.4</v>
+        <v>148092.4</v>
       </c>
       <c r="P36" s="7" t="n">
-        <v>11.72140993359866</v>
+        <v>12.29475651687731</v>
       </c>
       <c r="Q36" s="8" t="inlineStr"/>
       <c r="R36" s="8" t="inlineStr"/>
       <c r="S36" s="6" t="n">
-        <v>134467.16</v>
+        <v>133383.16</v>
       </c>
       <c r="T36" s="7" t="n">
-        <v>23.67331919555674</v>
+        <v>24.67840767905033</v>
       </c>
       <c r="U36" s="8" t="inlineStr"/>
       <c r="V36" s="8" t="inlineStr"/>
@@ -3451,7 +3451,7 @@
       <c r="AD36" s="8" t="inlineStr"/>
       <c r="AE36" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:38</t>
+          <t>2025-10-18 11:05:50</t>
         </is>
       </c>
       <c r="AF36" s="8" t="inlineStr"/>
@@ -3531,7 +3531,7 @@
       <c r="AD37" s="8" t="inlineStr"/>
       <c r="AE37" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:39</t>
+          <t>2025-10-18 11:05:51</t>
         </is>
       </c>
       <c r="AF37" s="8" t="inlineStr"/>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 7.5% (접근 중!)</t>
+          <t>1차 매수선까지 7.7% (접근 중!)</t>
         </is>
       </c>
       <c r="F38" s="6" t="n">
@@ -3578,26 +3578,26 @@
         <v>19864</v>
       </c>
       <c r="K38" s="6" t="n">
-        <v>19914</v>
+        <v>19874</v>
       </c>
       <c r="L38" s="7" t="n">
-        <v>7.46208697398815</v>
+        <v>7.678373754654322</v>
       </c>
       <c r="M38" s="8" t="inlineStr"/>
       <c r="N38" s="8" t="inlineStr"/>
       <c r="O38" s="6" t="n">
-        <v>17972.6</v>
+        <v>17896.6</v>
       </c>
       <c r="P38" s="7" t="n">
-        <v>19.07014010215549</v>
+        <v>19.57578534470233</v>
       </c>
       <c r="Q38" s="8" t="inlineStr"/>
       <c r="R38" s="8" t="inlineStr"/>
       <c r="S38" s="6" t="n">
-        <v>16225.34</v>
+        <v>16116.94</v>
       </c>
       <c r="T38" s="7" t="n">
-        <v>31.89245957249585</v>
+        <v>32.77954748233844</v>
       </c>
       <c r="U38" s="8" t="inlineStr"/>
       <c r="V38" s="8" t="inlineStr"/>
@@ -3611,7 +3611,7 @@
       <c r="AD38" s="8" t="inlineStr"/>
       <c r="AE38" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:39</t>
+          <t>2025-10-18 11:05:51</t>
         </is>
       </c>
       <c r="AF38" s="8" t="inlineStr"/>
@@ -3674,10 +3674,10 @@
       <c r="Q39" s="8" t="inlineStr"/>
       <c r="R39" s="8" t="inlineStr"/>
       <c r="S39" s="6" t="n">
-        <v>18112.64</v>
+        <v>18072.64</v>
       </c>
       <c r="T39" s="7" t="n">
-        <v>41.61381223278327</v>
+        <v>41.92724471908916</v>
       </c>
       <c r="U39" s="8" t="inlineStr"/>
       <c r="V39" s="8" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       <c r="AD39" s="8" t="inlineStr"/>
       <c r="AE39" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:39</t>
+          <t>2025-10-18 11:05:51</t>
         </is>
       </c>
       <c r="AF39" s="8" t="inlineStr"/>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 16.0%</t>
+          <t>1차 매수선까지 16.3%</t>
         </is>
       </c>
       <c r="F40" s="6" t="n">
@@ -3738,26 +3738,26 @@
         <v>17275.6</v>
       </c>
       <c r="K40" s="6" t="n">
-        <v>17325.6</v>
+        <v>17285.6</v>
       </c>
       <c r="L40" s="7" t="n">
-        <v>16.01329824075355</v>
+        <v>16.28176054056554</v>
       </c>
       <c r="M40" s="8" t="inlineStr"/>
       <c r="N40" s="8" t="inlineStr"/>
       <c r="O40" s="6" t="n">
-        <v>15643.04</v>
+        <v>15567.04</v>
       </c>
       <c r="P40" s="7" t="n">
-        <v>28.49164868209758</v>
+        <v>29.11895903138937</v>
       </c>
       <c r="Q40" s="8" t="inlineStr"/>
       <c r="R40" s="8" t="inlineStr"/>
       <c r="S40" s="6" t="n">
-        <v>14128.736</v>
+        <v>14020.336</v>
       </c>
       <c r="T40" s="7" t="n">
-        <v>42.26325695377135</v>
+        <v>43.36318330744709</v>
       </c>
       <c r="U40" s="8" t="inlineStr"/>
       <c r="V40" s="8" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
       <c r="AD40" s="8" t="inlineStr"/>
       <c r="AE40" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:40</t>
+          <t>2025-10-18 11:05:52</t>
         </is>
       </c>
       <c r="AF40" s="8" t="inlineStr"/>
@@ -3851,7 +3851,7 @@
       <c r="AD41" s="8" t="inlineStr"/>
       <c r="AE41" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:40</t>
+          <t>2025-10-18 11:05:52</t>
         </is>
       </c>
       <c r="AF41" s="8" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       <c r="AD42" s="8" t="inlineStr"/>
       <c r="AE42" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:40</t>
+          <t>2025-10-18 11:05:52</t>
         </is>
       </c>
       <c r="AF42" s="8" t="inlineStr"/>
@@ -3986,18 +3986,18 @@
       <c r="M43" s="8" t="inlineStr"/>
       <c r="N43" s="8" t="inlineStr"/>
       <c r="O43" s="6" t="n">
-        <v>18573.8</v>
+        <v>18533.8</v>
       </c>
       <c r="P43" s="7" t="n">
-        <v>21.40757410976753</v>
+        <v>21.66959824752615</v>
       </c>
       <c r="Q43" s="8" t="inlineStr"/>
       <c r="R43" s="8" t="inlineStr"/>
       <c r="S43" s="6" t="n">
-        <v>16766.42</v>
+        <v>16690.42</v>
       </c>
       <c r="T43" s="7" t="n">
-        <v>34.49502040387872</v>
+        <v>35.1074448695719</v>
       </c>
       <c r="U43" s="8" t="inlineStr"/>
       <c r="V43" s="8" t="inlineStr"/>
@@ -4011,7 +4011,7 @@
       <c r="AD43" s="8" t="inlineStr"/>
       <c r="AE43" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:41</t>
+          <t>2025-10-18 11:05:53</t>
         </is>
       </c>
       <c r="AF43" s="8" t="inlineStr"/>
@@ -4091,7 +4091,7 @@
       <c r="AD44" s="8" t="inlineStr"/>
       <c r="AE44" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:41</t>
+          <t>2025-10-18 11:05:53</t>
         </is>
       </c>
       <c r="AF44" s="8" t="inlineStr"/>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 24.7%</t>
+          <t>1차 매수선까지 25.0%</t>
         </is>
       </c>
       <c r="F45" s="6" t="n">
@@ -4138,26 +4138,26 @@
         <v>159452</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>159952</v>
+        <v>159552</v>
       </c>
       <c r="L45" s="7" t="n">
-        <v>24.72491747524257</v>
+        <v>25.03760529482551</v>
       </c>
       <c r="M45" s="8" t="inlineStr"/>
       <c r="N45" s="8" t="inlineStr"/>
       <c r="O45" s="6" t="n">
-        <v>144456.8</v>
+        <v>143696.8</v>
       </c>
       <c r="P45" s="7" t="n">
-        <v>38.10357144834994</v>
+        <v>38.83398934423033</v>
       </c>
       <c r="Q45" s="8" t="inlineStr"/>
       <c r="R45" s="8" t="inlineStr"/>
       <c r="S45" s="6" t="n">
-        <v>130511.12</v>
+        <v>129427.12</v>
       </c>
       <c r="T45" s="7" t="n">
-        <v>52.86053786068188</v>
+        <v>54.14080140236448</v>
       </c>
       <c r="U45" s="8" t="inlineStr"/>
       <c r="V45" s="8" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       <c r="AD45" s="8" t="inlineStr"/>
       <c r="AE45" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:41</t>
+          <t>2025-10-18 11:05:53</t>
         </is>
       </c>
       <c r="AF45" s="8" t="inlineStr"/>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 27.5%</t>
+          <t>1차 매수선까지 27.7%</t>
         </is>
       </c>
       <c r="F46" s="6" t="n">
@@ -4218,26 +4218,26 @@
         <v>17368</v>
       </c>
       <c r="K46" s="6" t="n">
-        <v>17418</v>
+        <v>17378</v>
       </c>
       <c r="L46" s="7" t="n">
-        <v>27.45435756114365</v>
+        <v>27.74772701116354</v>
       </c>
       <c r="M46" s="8" t="inlineStr"/>
       <c r="N46" s="8" t="inlineStr"/>
       <c r="O46" s="6" t="n">
-        <v>15726.2</v>
+        <v>15650.2</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>41.1656980071473</v>
+        <v>41.85122234859618</v>
       </c>
       <c r="Q46" s="8" t="inlineStr"/>
       <c r="R46" s="8" t="inlineStr"/>
       <c r="S46" s="6" t="n">
-        <v>14203.58</v>
+        <v>14095.18</v>
       </c>
       <c r="T46" s="7" t="n">
-        <v>56.29862330482877</v>
+        <v>57.50064915808098</v>
       </c>
       <c r="U46" s="8" t="inlineStr"/>
       <c r="V46" s="8" t="inlineStr"/>
@@ -4251,7 +4251,7 @@
       <c r="AD46" s="8" t="inlineStr"/>
       <c r="AE46" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:42</t>
+          <t>2025-10-18 11:05:54</t>
         </is>
       </c>
       <c r="AF46" s="8" t="inlineStr"/>
@@ -4331,7 +4331,7 @@
       <c r="AD47" s="8" t="inlineStr"/>
       <c r="AE47" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:42</t>
+          <t>2025-10-18 11:05:54</t>
         </is>
       </c>
       <c r="AF47" s="8" t="inlineStr"/>
@@ -4411,7 +4411,7 @@
       <c r="AD48" s="8" t="inlineStr"/>
       <c r="AE48" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:42</t>
+          <t>2025-10-18 11:05:54</t>
         </is>
       </c>
       <c r="AF48" s="8" t="inlineStr"/>
@@ -4491,7 +4491,7 @@
       <c r="AD49" s="8" t="inlineStr"/>
       <c r="AE49" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:43</t>
+          <t>2025-10-18 11:05:55</t>
         </is>
       </c>
       <c r="AF49" s="8" t="inlineStr"/>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 7.7% (접근 중!)</t>
+          <t>1차 매수선까지 8.0% (접근 중!)</t>
         </is>
       </c>
       <c r="F50" s="6" t="n">
@@ -4538,26 +4538,26 @@
         <v>14830</v>
       </c>
       <c r="K50" s="6" t="n">
-        <v>14880</v>
+        <v>14840</v>
       </c>
       <c r="L50" s="7" t="n">
-        <v>7.661290322580645</v>
+        <v>7.951482479784366</v>
       </c>
       <c r="M50" s="8" t="inlineStr"/>
       <c r="N50" s="8" t="inlineStr"/>
       <c r="O50" s="6" t="n">
-        <v>13442</v>
+        <v>13366</v>
       </c>
       <c r="P50" s="7" t="n">
-        <v>19.17869364677875</v>
+        <v>19.85635193775251</v>
       </c>
       <c r="Q50" s="8" t="inlineStr"/>
       <c r="R50" s="8" t="inlineStr"/>
       <c r="S50" s="6" t="n">
-        <v>12147.8</v>
+        <v>12039.4</v>
       </c>
       <c r="T50" s="7" t="n">
-        <v>31.87573058496188</v>
+        <v>33.06310945728193</v>
       </c>
       <c r="U50" s="8" t="inlineStr"/>
       <c r="V50" s="8" t="inlineStr"/>
@@ -4571,7 +4571,7 @@
       <c r="AD50" s="8" t="inlineStr"/>
       <c r="AE50" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:43</t>
+          <t>2025-10-18 11:05:55</t>
         </is>
       </c>
       <c r="AF50" s="8" t="inlineStr"/>
@@ -4651,7 +4651,7 @@
       <c r="AD51" s="8" t="inlineStr"/>
       <c r="AE51" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:43</t>
+          <t>2025-10-18 11:05:55</t>
         </is>
       </c>
       <c r="AF51" s="8" t="inlineStr"/>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 26.4%</t>
+          <t>1차 매수선까지 26.9%</t>
         </is>
       </c>
       <c r="F52" s="6" t="n">
@@ -4698,26 +4698,26 @@
         <v>11183.6</v>
       </c>
       <c r="K52" s="6" t="n">
-        <v>11233.6</v>
+        <v>11193.6</v>
       </c>
       <c r="L52" s="7" t="n">
-        <v>26.40649480131035</v>
+        <v>26.85820468839336</v>
       </c>
       <c r="M52" s="8" t="inlineStr"/>
       <c r="N52" s="8" t="inlineStr"/>
       <c r="O52" s="6" t="n">
-        <v>10160.24</v>
+        <v>10084.24</v>
       </c>
       <c r="P52" s="7" t="n">
-        <v>39.76047809894255</v>
+        <v>40.81378467787359</v>
       </c>
       <c r="Q52" s="8" t="inlineStr"/>
       <c r="R52" s="8" t="inlineStr"/>
       <c r="S52" s="6" t="n">
-        <v>9154.216</v>
+        <v>9085.816000000001</v>
       </c>
       <c r="T52" s="7" t="n">
-        <v>55.11978305952142</v>
+        <v>56.28755854179744</v>
       </c>
       <c r="U52" s="8" t="inlineStr"/>
       <c r="V52" s="8" t="inlineStr"/>
@@ -4731,7 +4731,7 @@
       <c r="AD52" s="8" t="inlineStr"/>
       <c r="AE52" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:44</t>
+          <t>2025-10-18 11:05:56</t>
         </is>
       </c>
       <c r="AF52" s="8" t="inlineStr"/>
@@ -4811,7 +4811,7 @@
       <c r="AD53" s="8" t="inlineStr"/>
       <c r="AE53" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:44</t>
+          <t>2025-10-18 11:05:56</t>
         </is>
       </c>
       <c r="AF53" s="8" t="inlineStr"/>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 25.6%</t>
+          <t>1차 매수선까지 25.9%</t>
         </is>
       </c>
       <c r="F54" s="6" t="n">
@@ -4858,26 +4858,26 @@
         <v>188160</v>
       </c>
       <c r="K54" s="6" t="n">
-        <v>188660</v>
+        <v>188260</v>
       </c>
       <c r="L54" s="7" t="n">
-        <v>25.62281352697975</v>
+        <v>25.88972697333475</v>
       </c>
       <c r="M54" s="8" t="inlineStr"/>
       <c r="N54" s="8" t="inlineStr"/>
       <c r="O54" s="6" t="n">
-        <v>170294</v>
+        <v>169534</v>
       </c>
       <c r="P54" s="7" t="n">
-        <v>39.1710806017828</v>
+        <v>39.79496738117428</v>
       </c>
       <c r="Q54" s="8" t="inlineStr"/>
       <c r="R54" s="8" t="inlineStr"/>
       <c r="S54" s="6" t="n">
-        <v>153764.6</v>
+        <v>152680.6</v>
       </c>
       <c r="T54" s="7" t="n">
-        <v>54.13170521693549</v>
+        <v>55.22600775737061</v>
       </c>
       <c r="U54" s="8" t="inlineStr"/>
       <c r="V54" s="8" t="inlineStr"/>
@@ -4891,7 +4891,7 @@
       <c r="AD54" s="8" t="inlineStr"/>
       <c r="AE54" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:44</t>
+          <t>2025-10-18 11:05:56</t>
         </is>
       </c>
       <c r="AF54" s="8" t="inlineStr"/>
@@ -4971,7 +4971,7 @@
       <c r="AD55" s="8" t="inlineStr"/>
       <c r="AE55" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:44</t>
+          <t>2025-10-18 11:05:57</t>
         </is>
       </c>
       <c r="AF55" s="8" t="inlineStr"/>
@@ -5051,7 +5051,7 @@
       <c r="AD56" s="8" t="inlineStr"/>
       <c r="AE56" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:45</t>
+          <t>2025-10-18 11:05:57</t>
         </is>
       </c>
       <c r="AF56" s="8" t="inlineStr"/>
@@ -5131,7 +5131,7 @@
       <c r="AD57" s="8" t="inlineStr"/>
       <c r="AE57" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:45</t>
+          <t>2025-10-18 11:05:57</t>
         </is>
       </c>
       <c r="AF57" s="8" t="inlineStr"/>
@@ -5194,10 +5194,10 @@
       <c r="Q58" s="8" t="inlineStr"/>
       <c r="R58" s="8" t="inlineStr"/>
       <c r="S58" s="6" t="n">
-        <v>19076.54</v>
+        <v>19036.54</v>
       </c>
       <c r="T58" s="7" t="n">
-        <v>54.11599797447545</v>
+        <v>54.43982992707708</v>
       </c>
       <c r="U58" s="8" t="inlineStr"/>
       <c r="V58" s="8" t="inlineStr"/>
@@ -5211,7 +5211,7 @@
       <c r="AD58" s="8" t="inlineStr"/>
       <c r="AE58" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:45</t>
+          <t>2025-10-18 11:05:58</t>
         </is>
       </c>
       <c r="AF58" s="8" t="inlineStr"/>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 27.2%</t>
+          <t>1차 매수선까지 27.6%</t>
         </is>
       </c>
       <c r="F59" s="6" t="n">
@@ -5258,26 +5258,26 @@
         <v>158640</v>
       </c>
       <c r="K59" s="6" t="n">
-        <v>159140</v>
+        <v>158740</v>
       </c>
       <c r="L59" s="7" t="n">
-        <v>27.24644966695991</v>
+        <v>27.5670908403679</v>
       </c>
       <c r="M59" s="8" t="inlineStr"/>
       <c r="N59" s="8" t="inlineStr"/>
       <c r="O59" s="6" t="n">
-        <v>143726</v>
+        <v>142966</v>
       </c>
       <c r="P59" s="7" t="n">
-        <v>40.8930882373405</v>
+        <v>41.64206874361736</v>
       </c>
       <c r="Q59" s="8" t="inlineStr"/>
       <c r="R59" s="8" t="inlineStr"/>
       <c r="S59" s="6" t="n">
-        <v>129853.4</v>
+        <v>128769.4</v>
       </c>
       <c r="T59" s="7" t="n">
-        <v>55.94508884634518</v>
+        <v>57.25785784510915</v>
       </c>
       <c r="U59" s="8" t="inlineStr"/>
       <c r="V59" s="8" t="inlineStr"/>
@@ -5291,7 +5291,7 @@
       <c r="AD59" s="8" t="inlineStr"/>
       <c r="AE59" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:46</t>
+          <t>2025-10-18 11:05:58</t>
         </is>
       </c>
       <c r="AF59" s="8" t="inlineStr"/>
@@ -5371,7 +5371,7 @@
       <c r="AD60" s="8" t="inlineStr"/>
       <c r="AE60" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:46</t>
+          <t>2025-10-18 11:05:58</t>
         </is>
       </c>
       <c r="AF60" s="8" t="inlineStr"/>
@@ -5399,7 +5399,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 18.7%</t>
+          <t>1차 매수선까지 19.1%</t>
         </is>
       </c>
       <c r="F61" s="6" t="n">
@@ -5418,26 +5418,26 @@
         <v>12316.8</v>
       </c>
       <c r="K61" s="6" t="n">
-        <v>12366.8</v>
+        <v>12326.8</v>
       </c>
       <c r="L61" s="7" t="n">
-        <v>18.70491962350809</v>
+        <v>19.0901126001882</v>
       </c>
       <c r="M61" s="8" t="inlineStr"/>
       <c r="N61" s="8" t="inlineStr"/>
       <c r="O61" s="6" t="n">
-        <v>11180.12</v>
+        <v>11104.12</v>
       </c>
       <c r="P61" s="7" t="n">
-        <v>31.30449404836441</v>
+        <v>32.20318224226683</v>
       </c>
       <c r="Q61" s="8" t="inlineStr"/>
       <c r="R61" s="8" t="inlineStr"/>
       <c r="S61" s="6" t="n">
-        <v>10112.108</v>
+        <v>10003.708</v>
       </c>
       <c r="T61" s="7" t="n">
-        <v>45.17250013548114</v>
+        <v>46.74558673643812</v>
       </c>
       <c r="U61" s="8" t="inlineStr"/>
       <c r="V61" s="8" t="inlineStr"/>
@@ -5451,7 +5451,7 @@
       <c r="AD61" s="8" t="inlineStr"/>
       <c r="AE61" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:46</t>
+          <t>2025-10-18 11:05:59</t>
         </is>
       </c>
       <c r="AF61" s="8" t="inlineStr"/>
@@ -5514,10 +5514,10 @@
       <c r="Q62" s="8" t="inlineStr"/>
       <c r="R62" s="8" t="inlineStr"/>
       <c r="S62" s="6" t="n">
-        <v>19844.42</v>
+        <v>19804.42</v>
       </c>
       <c r="T62" s="7" t="n">
-        <v>52.18383807639631</v>
+        <v>52.49121155782397</v>
       </c>
       <c r="U62" s="8" t="inlineStr"/>
       <c r="V62" s="8" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
       <c r="AD62" s="8" t="inlineStr"/>
       <c r="AE62" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:47</t>
+          <t>2025-10-18 11:05:59</t>
         </is>
       </c>
       <c r="AF62" s="8" t="inlineStr"/>
@@ -5586,18 +5586,18 @@
       <c r="M63" s="8" t="inlineStr"/>
       <c r="N63" s="8" t="inlineStr"/>
       <c r="O63" s="6" t="n">
-        <v>1901.84</v>
+        <v>1897.84</v>
       </c>
       <c r="P63" s="7" t="n">
-        <v>37.23551928658563</v>
+        <v>37.52476499599545</v>
       </c>
       <c r="Q63" s="8" t="inlineStr"/>
       <c r="R63" s="8" t="inlineStr"/>
       <c r="S63" s="6" t="n">
-        <v>1716.656</v>
+        <v>1709.056</v>
       </c>
       <c r="T63" s="7" t="n">
-        <v>52.03977966465034</v>
+        <v>52.71588526063511</v>
       </c>
       <c r="U63" s="8" t="inlineStr"/>
       <c r="V63" s="8" t="inlineStr"/>
@@ -5611,7 +5611,7 @@
       <c r="AD63" s="8" t="inlineStr"/>
       <c r="AE63" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:47</t>
+          <t>2025-10-18 11:05:59</t>
         </is>
       </c>
       <c r="AF63" s="8" t="inlineStr"/>
@@ -5691,7 +5691,7 @@
       <c r="AD64" s="8" t="inlineStr"/>
       <c r="AE64" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:47</t>
+          <t>2025-10-18 11:06:00</t>
         </is>
       </c>
       <c r="AF64" s="8" t="inlineStr"/>
@@ -5714,12 +5714,12 @@
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>READY_BUY1</t>
+          <t>WATCHING</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 10.0% (접근 중!)</t>
+          <t>1차 매수선까지 10.4%</t>
         </is>
       </c>
       <c r="F65" s="6" t="n">
@@ -5738,26 +5738,26 @@
         <v>118064</v>
       </c>
       <c r="K65" s="6" t="n">
-        <v>118564</v>
+        <v>118164</v>
       </c>
       <c r="L65" s="7" t="n">
-        <v>9.982794102763066</v>
+        <v>10.35509969195356</v>
       </c>
       <c r="M65" s="8" t="inlineStr"/>
       <c r="N65" s="8" t="inlineStr"/>
       <c r="O65" s="6" t="n">
-        <v>107207.6</v>
+        <v>106447.6</v>
       </c>
       <c r="P65" s="7" t="n">
-        <v>21.63316779780537</v>
+        <v>22.50158763560662</v>
       </c>
       <c r="Q65" s="8" t="inlineStr"/>
       <c r="R65" s="8" t="inlineStr"/>
       <c r="S65" s="6" t="n">
-        <v>96586.84000000001</v>
+        <v>95902.84000000001</v>
       </c>
       <c r="T65" s="7" t="n">
-        <v>35.00804043283742</v>
+        <v>35.97094726287562</v>
       </c>
       <c r="U65" s="8" t="inlineStr"/>
       <c r="V65" s="8" t="inlineStr"/>
@@ -5771,7 +5771,7 @@
       <c r="AD65" s="8" t="inlineStr"/>
       <c r="AE65" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:48</t>
+          <t>2025-10-18 11:06:00</t>
         </is>
       </c>
       <c r="AF65" s="8" t="inlineStr"/>
@@ -5851,7 +5851,7 @@
       <c r="AD66" s="8" t="inlineStr"/>
       <c r="AE66" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:48</t>
+          <t>2025-10-18 11:06:00</t>
         </is>
       </c>
       <c r="AF66" s="8" t="inlineStr"/>
@@ -5931,7 +5931,7 @@
       <c r="AD67" s="8" t="inlineStr"/>
       <c r="AE67" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:49</t>
+          <t>2025-10-18 11:06:01</t>
         </is>
       </c>
       <c r="AF67" s="8" t="inlineStr"/>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="E68" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 44.4%</t>
+          <t>1차 매수선까지 44.7%</t>
         </is>
       </c>
       <c r="F68" s="6" t="n">
@@ -5978,26 +5978,26 @@
         <v>176796</v>
       </c>
       <c r="K68" s="6" t="n">
-        <v>177296</v>
+        <v>176896</v>
       </c>
       <c r="L68" s="7" t="n">
-        <v>44.39130042414944</v>
+        <v>44.7178002894356</v>
       </c>
       <c r="M68" s="8" t="inlineStr"/>
       <c r="N68" s="8" t="inlineStr"/>
       <c r="O68" s="6" t="n">
-        <v>160066.4</v>
+        <v>159306.4</v>
       </c>
       <c r="P68" s="7" t="n">
-        <v>59.93362754456901</v>
+        <v>60.69661984703691</v>
       </c>
       <c r="Q68" s="8" t="inlineStr"/>
       <c r="R68" s="8" t="inlineStr"/>
       <c r="S68" s="6" t="n">
-        <v>144559.76</v>
+        <v>143475.76</v>
       </c>
       <c r="T68" s="7" t="n">
-        <v>77.08939195803866</v>
+        <v>78.42735246706481</v>
       </c>
       <c r="U68" s="8" t="inlineStr"/>
       <c r="V68" s="8" t="inlineStr"/>
@@ -6011,7 +6011,7 @@
       <c r="AD68" s="8" t="inlineStr"/>
       <c r="AE68" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:49</t>
+          <t>2025-10-18 11:06:01</t>
         </is>
       </c>
       <c r="AF68" s="8" t="inlineStr"/>
@@ -6074,10 +6074,10 @@
       <c r="Q69" s="8" t="inlineStr"/>
       <c r="R69" s="8" t="inlineStr"/>
       <c r="S69" s="6" t="n">
-        <v>182373.8</v>
+        <v>181973.8</v>
       </c>
       <c r="T69" s="7" t="n">
-        <v>58.46574453128682</v>
+        <v>58.81407103659976</v>
       </c>
       <c r="U69" s="8" t="inlineStr"/>
       <c r="V69" s="8" t="inlineStr"/>
@@ -6091,7 +6091,7 @@
       <c r="AD69" s="8" t="inlineStr"/>
       <c r="AE69" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:49</t>
+          <t>2025-10-18 11:06:01</t>
         </is>
       </c>
       <c r="AF69" s="8" t="inlineStr"/>
@@ -6171,7 +6171,7 @@
       <c r="AD70" s="8" t="inlineStr"/>
       <c r="AE70" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:50</t>
+          <t>2025-10-18 11:06:02</t>
         </is>
       </c>
       <c r="AF70" s="8" t="inlineStr"/>
@@ -6251,7 +6251,7 @@
       <c r="AD71" s="8" t="inlineStr"/>
       <c r="AE71" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:50</t>
+          <t>2025-10-18 11:06:02</t>
         </is>
       </c>
       <c r="AF71" s="8" t="inlineStr"/>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 22.2%</t>
+          <t>1차 매수선까지 22.5%</t>
         </is>
       </c>
       <c r="F72" s="6" t="n">
@@ -6298,26 +6298,26 @@
         <v>176600</v>
       </c>
       <c r="K72" s="6" t="n">
-        <v>177100</v>
+        <v>176700</v>
       </c>
       <c r="L72" s="7" t="n">
-        <v>22.24731789949181</v>
+        <v>22.52405206564799</v>
       </c>
       <c r="M72" s="8" t="inlineStr"/>
       <c r="N72" s="8" t="inlineStr"/>
       <c r="O72" s="6" t="n">
-        <v>159890</v>
+        <v>159130</v>
       </c>
       <c r="P72" s="7" t="n">
-        <v>35.40559134404903</v>
+        <v>36.05228429585873</v>
       </c>
       <c r="Q72" s="8" t="inlineStr"/>
       <c r="R72" s="8" t="inlineStr"/>
       <c r="S72" s="6" t="n">
-        <v>144401</v>
+        <v>143317</v>
       </c>
       <c r="T72" s="7" t="n">
-        <v>49.92970962804966</v>
+        <v>51.06372586643594</v>
       </c>
       <c r="U72" s="8" t="inlineStr"/>
       <c r="V72" s="8" t="inlineStr"/>
@@ -6331,7 +6331,7 @@
       <c r="AD72" s="8" t="inlineStr"/>
       <c r="AE72" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:50</t>
+          <t>2025-10-18 11:06:02</t>
         </is>
       </c>
       <c r="AF72" s="8" t="inlineStr"/>
@@ -6411,7 +6411,7 @@
       <c r="AD73" s="8" t="inlineStr"/>
       <c r="AE73" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 10:45:51</t>
+          <t>2025-10-18 11:06:03</t>
         </is>
       </c>
       <c r="AF73" s="8" t="inlineStr"/>

</xml_diff>

<commit_message>
Fix tick calculation to always use upper tick price
- Trading_Signal_System.py: Updated get_nearest_tick_price function
  - Changed from 'closest tick' to 'always upper tick' logic
  - When price is between lower and upper tick, always choose upper tick
  - No distance comparison, always rounds up to next valid tick

- Real_Time_Monitor.py: Updated get_nearest_tick_price function
  - Applied same 'always upper tick' logic
  - Consistent with Trading_Signal_System.py

- Key improvements:
  - SK Hynix: 301,860????302,000??(500??tick)
  - Doosan Energy: 55,052????55,100??(100??tick)
  - Samsung Electronics: 69,344????69,400??(100??tick)
  - NAVER: 200,740????201,000??(500??tick)
  - User example: 95,431????95,500??(100??tick)

- All buy lines now represent actual purchasable upper tick prices
- Follows user requirement: 'current price between ticks ??always upper tick'
- Tested successfully with force execution mode
</commit_message>
<xml_diff>
--- a/output/trading_signals.xlsx
+++ b/output/trading_signals.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="AH1" s="3" t="inlineStr">
         <is>
-          <t>최종 업데이트: 2025-10-18 11:08:39</t>
+          <t>최종 업데이트: 2025-10-18 11:11:39</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 39.0%</t>
+          <t>1차 매수선까지 38.8%</t>
         </is>
       </c>
       <c r="F2" s="6" t="n">
@@ -698,26 +698,26 @@
         <v>69244</v>
       </c>
       <c r="K2" s="6" t="n">
-        <v>69300</v>
+        <v>69400</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>38.96103896103897</v>
+        <v>38.76080691642652</v>
       </c>
       <c r="M2" s="8" t="inlineStr"/>
       <c r="N2" s="8" t="inlineStr"/>
       <c r="O2" s="6" t="n">
-        <v>62500</v>
+        <v>62600</v>
       </c>
       <c r="P2" s="7" t="n">
-        <v>54.08</v>
+        <v>53.83386581469649</v>
       </c>
       <c r="Q2" s="8" t="inlineStr"/>
       <c r="R2" s="8" t="inlineStr"/>
       <c r="S2" s="6" t="n">
-        <v>56300</v>
+        <v>56500</v>
       </c>
       <c r="T2" s="7" t="n">
-        <v>71.04795737122558</v>
+        <v>70.4424778761062</v>
       </c>
       <c r="U2" s="8" t="inlineStr"/>
       <c r="V2" s="8" t="inlineStr"/>
@@ -731,7 +731,7 @@
       <c r="AD2" s="8" t="inlineStr"/>
       <c r="AE2" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:18</t>
+          <t>2025-10-18 11:11:16</t>
         </is>
       </c>
       <c r="AF2" s="8" t="inlineStr"/>
@@ -794,10 +794,10 @@
       <c r="Q3" s="8" t="inlineStr"/>
       <c r="R3" s="8" t="inlineStr"/>
       <c r="S3" s="6" t="n">
-        <v>245500</v>
+        <v>246000</v>
       </c>
       <c r="T3" s="7" t="n">
-        <v>85.13238289205702</v>
+        <v>84.7560975609756</v>
       </c>
       <c r="U3" s="8" t="inlineStr"/>
       <c r="V3" s="8" t="inlineStr"/>
@@ -811,7 +811,7 @@
       <c r="AD3" s="8" t="inlineStr"/>
       <c r="AE3" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:19</t>
+          <t>2025-10-18 11:11:16</t>
         </is>
       </c>
       <c r="AF3" s="8" t="inlineStr"/>
@@ -839,7 +839,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 46.9%</t>
+          <t>1차 매수선까지 46.6%</t>
         </is>
       </c>
       <c r="F4" s="6" t="n">
@@ -858,26 +858,26 @@
         <v>54128</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>54200</v>
+        <v>54300</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>46.86346863468634</v>
+        <v>46.59300184162063</v>
       </c>
       <c r="M4" s="8" t="inlineStr"/>
       <c r="N4" s="8" t="inlineStr"/>
       <c r="O4" s="6" t="n">
-        <v>48850</v>
+        <v>48950</v>
       </c>
       <c r="P4" s="7" t="n">
-        <v>62.94779938587512</v>
+        <v>62.61491317671093</v>
       </c>
       <c r="Q4" s="8" t="inlineStr"/>
       <c r="R4" s="8" t="inlineStr"/>
       <c r="S4" s="6" t="n">
-        <v>44000</v>
+        <v>44150</v>
       </c>
       <c r="T4" s="7" t="n">
-        <v>80.90909090909091</v>
+        <v>80.29445073612685</v>
       </c>
       <c r="U4" s="8" t="inlineStr"/>
       <c r="V4" s="8" t="inlineStr"/>
@@ -891,7 +891,7 @@
       <c r="AD4" s="8" t="inlineStr"/>
       <c r="AE4" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:19</t>
+          <t>2025-10-18 11:11:17</t>
         </is>
       </c>
       <c r="AF4" s="8" t="inlineStr"/>
@@ -946,18 +946,18 @@
       <c r="M5" s="8" t="inlineStr"/>
       <c r="N5" s="8" t="inlineStr"/>
       <c r="O5" s="6" t="n">
-        <v>179900</v>
+        <v>180000</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>39.24402445803224</v>
+        <v>39.16666666666666</v>
       </c>
       <c r="Q5" s="8" t="inlineStr"/>
       <c r="R5" s="8" t="inlineStr"/>
       <c r="S5" s="6" t="n">
-        <v>162000</v>
+        <v>162100</v>
       </c>
       <c r="T5" s="7" t="n">
-        <v>54.62962962962963</v>
+        <v>54.53423812461443</v>
       </c>
       <c r="U5" s="8" t="inlineStr"/>
       <c r="V5" s="8" t="inlineStr"/>
@@ -971,7 +971,7 @@
       <c r="AD5" s="8" t="inlineStr"/>
       <c r="AE5" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:20</t>
+          <t>2025-10-18 11:11:17</t>
         </is>
       </c>
       <c r="AF5" s="8" t="inlineStr"/>
@@ -1034,10 +1034,10 @@
       <c r="Q6" s="8" t="inlineStr"/>
       <c r="R6" s="8" t="inlineStr"/>
       <c r="S6" s="6" t="n">
-        <v>69000</v>
+        <v>69100</v>
       </c>
       <c r="T6" s="7" t="n">
-        <v>102.1739130434783</v>
+        <v>101.8813314037627</v>
       </c>
       <c r="U6" s="8" t="inlineStr"/>
       <c r="V6" s="8" t="inlineStr"/>
@@ -1051,7 +1051,7 @@
       <c r="AD6" s="8" t="inlineStr"/>
       <c r="AE6" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:20</t>
+          <t>2025-10-18 11:11:18</t>
         </is>
       </c>
       <c r="AF6" s="8" t="inlineStr"/>
@@ -1114,10 +1114,10 @@
       <c r="Q7" s="8" t="inlineStr"/>
       <c r="R7" s="8" t="inlineStr"/>
       <c r="S7" s="6" t="n">
-        <v>79000</v>
+        <v>79100</v>
       </c>
       <c r="T7" s="7" t="n">
-        <v>93.54430379746836</v>
+        <v>93.29962073324906</v>
       </c>
       <c r="U7" s="8" t="inlineStr"/>
       <c r="V7" s="8" t="inlineStr"/>
@@ -1131,7 +1131,7 @@
       <c r="AD7" s="8" t="inlineStr"/>
       <c r="AE7" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:20</t>
+          <t>2025-10-18 11:11:18</t>
         </is>
       </c>
       <c r="AF7" s="8" t="inlineStr"/>
@@ -1194,10 +1194,10 @@
       <c r="Q8" s="8" t="inlineStr"/>
       <c r="R8" s="8" t="inlineStr"/>
       <c r="S8" s="6" t="n">
-        <v>137500</v>
+        <v>137600</v>
       </c>
       <c r="T8" s="7" t="n">
-        <v>81.09090909090909</v>
+        <v>80.95930232558139</v>
       </c>
       <c r="U8" s="8" t="inlineStr"/>
       <c r="V8" s="8" t="inlineStr"/>
@@ -1211,7 +1211,7 @@
       <c r="AD8" s="8" t="inlineStr"/>
       <c r="AE8" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:21</t>
+          <t>2025-10-18 11:11:18</t>
         </is>
       </c>
       <c r="AF8" s="8" t="inlineStr"/>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 74.4%</t>
+          <t>1차 매수선까지 74.2%</t>
         </is>
       </c>
       <c r="F9" s="6" t="n">
@@ -1258,26 +1258,26 @@
         <v>40572</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>40600</v>
+        <v>40650</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>74.38423645320196</v>
+        <v>74.16974169741697</v>
       </c>
       <c r="M9" s="8" t="inlineStr"/>
       <c r="N9" s="8" t="inlineStr"/>
       <c r="O9" s="6" t="n">
-        <v>36600</v>
+        <v>36650</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>93.44262295081968</v>
+        <v>93.17871759890861</v>
       </c>
       <c r="Q9" s="8" t="inlineStr"/>
       <c r="R9" s="8" t="inlineStr"/>
       <c r="S9" s="6" t="n">
-        <v>33000</v>
+        <v>33050</v>
       </c>
       <c r="T9" s="7" t="n">
-        <v>114.5454545454545</v>
+        <v>114.2208774583964</v>
       </c>
       <c r="U9" s="8" t="inlineStr"/>
       <c r="V9" s="8" t="inlineStr"/>
@@ -1291,7 +1291,7 @@
       <c r="AD9" s="8" t="inlineStr"/>
       <c r="AE9" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:21</t>
+          <t>2025-10-18 11:11:19</t>
         </is>
       </c>
       <c r="AF9" s="8" t="inlineStr"/>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 50.7%</t>
+          <t>1차 매수선까지 50.5%</t>
         </is>
       </c>
       <c r="F10" s="6" t="n">
@@ -1338,26 +1338,26 @@
         <v>40904</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>40950</v>
+        <v>41000</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>50.67155067155067</v>
+        <v>50.48780487804878</v>
       </c>
       <c r="M10" s="8" t="inlineStr"/>
       <c r="N10" s="8" t="inlineStr"/>
       <c r="O10" s="6" t="n">
-        <v>36900</v>
+        <v>36950</v>
       </c>
       <c r="P10" s="7" t="n">
-        <v>67.20867208672087</v>
+        <v>66.98240866035182</v>
       </c>
       <c r="Q10" s="8" t="inlineStr"/>
       <c r="R10" s="8" t="inlineStr"/>
       <c r="S10" s="6" t="n">
-        <v>33250</v>
+        <v>33350</v>
       </c>
       <c r="T10" s="7" t="n">
-        <v>85.56390977443608</v>
+        <v>85.00749625187406</v>
       </c>
       <c r="U10" s="8" t="inlineStr"/>
       <c r="V10" s="8" t="inlineStr"/>
@@ -1371,7 +1371,7 @@
       <c r="AD10" s="8" t="inlineStr"/>
       <c r="AE10" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:21</t>
+          <t>2025-10-18 11:11:19</t>
         </is>
       </c>
       <c r="AF10" s="8" t="inlineStr"/>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 44.8%</t>
+          <t>1차 매수선까지 44.6%</t>
         </is>
       </c>
       <c r="F11" s="6" t="n">
@@ -1418,26 +1418,26 @@
         <v>290680</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>291000</v>
+        <v>291500</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>44.84536082474227</v>
+        <v>44.59691252144082</v>
       </c>
       <c r="M11" s="8" t="inlineStr"/>
       <c r="N11" s="8" t="inlineStr"/>
       <c r="O11" s="6" t="n">
-        <v>262500</v>
+        <v>263000</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>60.57142857142858</v>
+        <v>60.26615969581749</v>
       </c>
       <c r="Q11" s="8" t="inlineStr"/>
       <c r="R11" s="8" t="inlineStr"/>
       <c r="S11" s="6" t="n">
-        <v>236500</v>
+        <v>237500</v>
       </c>
       <c r="T11" s="7" t="n">
-        <v>78.22410147991543</v>
+        <v>77.47368421052632</v>
       </c>
       <c r="U11" s="8" t="inlineStr"/>
       <c r="V11" s="8" t="inlineStr"/>
@@ -1451,7 +1451,7 @@
       <c r="AD11" s="8" t="inlineStr"/>
       <c r="AE11" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:21</t>
+          <t>2025-10-18 11:11:19</t>
         </is>
       </c>
       <c r="AF11" s="8" t="inlineStr"/>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 22.6%</t>
+          <t>1차 매수선까지 22.5%</t>
         </is>
       </c>
       <c r="F12" s="6" t="n">
@@ -1498,26 +1498,26 @@
         <v>87436</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>87500</v>
+        <v>87600</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>22.62857142857143</v>
+        <v>22.48858447488584</v>
       </c>
       <c r="M12" s="8" t="inlineStr"/>
       <c r="N12" s="8" t="inlineStr"/>
       <c r="O12" s="6" t="n">
-        <v>78900</v>
+        <v>79000</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>35.99493029150824</v>
+        <v>35.82278481012658</v>
       </c>
       <c r="Q12" s="8" t="inlineStr"/>
       <c r="R12" s="8" t="inlineStr"/>
       <c r="S12" s="6" t="n">
-        <v>71100</v>
+        <v>71200</v>
       </c>
       <c r="T12" s="7" t="n">
-        <v>50.91420534458509</v>
+        <v>50.70224719101124</v>
       </c>
       <c r="U12" s="8" t="inlineStr"/>
       <c r="V12" s="8" t="inlineStr"/>
@@ -1531,7 +1531,7 @@
       <c r="AD12" s="8" t="inlineStr"/>
       <c r="AE12" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:22</t>
+          <t>2025-10-18 11:11:20</t>
         </is>
       </c>
       <c r="AF12" s="8" t="inlineStr"/>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 41.4%</t>
+          <t>1차 매수선까지 41.1%</t>
         </is>
       </c>
       <c r="F13" s="6" t="n">
@@ -1578,26 +1578,26 @@
         <v>29570</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>29600</v>
+        <v>29650</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>41.38513513513514</v>
+        <v>41.14671163575042</v>
       </c>
       <c r="M13" s="8" t="inlineStr"/>
       <c r="N13" s="8" t="inlineStr"/>
       <c r="O13" s="6" t="n">
-        <v>26700</v>
+        <v>26750</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>56.74157303370787</v>
+        <v>56.44859813084112</v>
       </c>
       <c r="Q13" s="8" t="inlineStr"/>
       <c r="R13" s="8" t="inlineStr"/>
       <c r="S13" s="6" t="n">
-        <v>24100</v>
+        <v>24150</v>
       </c>
       <c r="T13" s="7" t="n">
-        <v>73.65145228215768</v>
+        <v>73.29192546583852</v>
       </c>
       <c r="U13" s="8" t="inlineStr"/>
       <c r="V13" s="8" t="inlineStr"/>
@@ -1611,7 +1611,7 @@
       <c r="AD13" s="8" t="inlineStr"/>
       <c r="AE13" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:22</t>
+          <t>2025-10-18 11:11:20</t>
         </is>
       </c>
       <c r="AF13" s="8" t="inlineStr"/>
@@ -1674,10 +1674,10 @@
       <c r="Q14" s="8" t="inlineStr"/>
       <c r="R14" s="8" t="inlineStr"/>
       <c r="S14" s="6" t="n">
-        <v>142800</v>
+        <v>142900</v>
       </c>
       <c r="T14" s="7" t="n">
-        <v>68.41736694677871</v>
+        <v>68.29951014695591</v>
       </c>
       <c r="U14" s="8" t="inlineStr"/>
       <c r="V14" s="8" t="inlineStr"/>
@@ -1691,7 +1691,7 @@
       <c r="AD14" s="8" t="inlineStr"/>
       <c r="AE14" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:22</t>
+          <t>2025-10-18 11:11:20</t>
         </is>
       </c>
       <c r="AF14" s="8" t="inlineStr"/>
@@ -1771,7 +1771,7 @@
       <c r="AD15" s="8" t="inlineStr"/>
       <c r="AE15" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:23</t>
+          <t>2025-10-18 11:11:21</t>
         </is>
       </c>
       <c r="AF15" s="8" t="inlineStr"/>
@@ -1799,7 +1799,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 66.9%</t>
+          <t>1차 매수선까지 66.7%</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
@@ -1818,26 +1818,26 @@
         <v>6820.400000000001</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>6830</v>
+        <v>6840</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>66.91068814055637</v>
+        <v>66.66666666666666</v>
       </c>
       <c r="M16" s="8" t="inlineStr"/>
       <c r="N16" s="8" t="inlineStr"/>
       <c r="O16" s="6" t="n">
-        <v>6160</v>
+        <v>6170</v>
       </c>
       <c r="P16" s="7" t="n">
-        <v>85.06493506493507</v>
+        <v>84.76499189627229</v>
       </c>
       <c r="Q16" s="8" t="inlineStr"/>
       <c r="R16" s="8" t="inlineStr"/>
       <c r="S16" s="6" t="n">
-        <v>5550</v>
+        <v>5570</v>
       </c>
       <c r="T16" s="7" t="n">
-        <v>105.4054054054054</v>
+        <v>104.6678635547576</v>
       </c>
       <c r="U16" s="8" t="inlineStr"/>
       <c r="V16" s="8" t="inlineStr"/>
@@ -1851,7 +1851,7 @@
       <c r="AD16" s="8" t="inlineStr"/>
       <c r="AE16" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:23</t>
+          <t>2025-10-18 11:11:21</t>
         </is>
       </c>
       <c r="AF16" s="8" t="inlineStr"/>
@@ -1906,18 +1906,18 @@
       <c r="M17" s="8" t="inlineStr"/>
       <c r="N17" s="8" t="inlineStr"/>
       <c r="O17" s="6" t="n">
-        <v>211500</v>
+        <v>212000</v>
       </c>
       <c r="P17" s="7" t="n">
-        <v>56.73758865248227</v>
+        <v>56.36792452830188</v>
       </c>
       <c r="Q17" s="8" t="inlineStr"/>
       <c r="R17" s="8" t="inlineStr"/>
       <c r="S17" s="6" t="n">
-        <v>190500</v>
+        <v>190900</v>
       </c>
       <c r="T17" s="7" t="n">
-        <v>74.01574803149606</v>
+        <v>73.65112624410686</v>
       </c>
       <c r="U17" s="8" t="inlineStr"/>
       <c r="V17" s="8" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
       <c r="AD17" s="8" t="inlineStr"/>
       <c r="AE17" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:23</t>
+          <t>2025-10-18 11:11:21</t>
         </is>
       </c>
       <c r="AF17" s="8" t="inlineStr"/>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 68.7%</t>
+          <t>1차 매수선까지 68.4%</t>
         </is>
       </c>
       <c r="F18" s="6" t="n">
@@ -1978,26 +1978,26 @@
         <v>62228</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>62300</v>
+        <v>62400</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>68.69983948635634</v>
+        <v>68.42948717948718</v>
       </c>
       <c r="M18" s="8" t="inlineStr"/>
       <c r="N18" s="8" t="inlineStr"/>
       <c r="O18" s="6" t="n">
-        <v>56200</v>
+        <v>56300</v>
       </c>
       <c r="P18" s="7" t="n">
-        <v>87.01067615658363</v>
+        <v>86.67850799289521</v>
       </c>
       <c r="Q18" s="8" t="inlineStr"/>
       <c r="R18" s="8" t="inlineStr"/>
       <c r="S18" s="6" t="n">
-        <v>50700</v>
+        <v>50800</v>
       </c>
       <c r="T18" s="7" t="n">
-        <v>107.2978303747534</v>
+        <v>106.8897637795276</v>
       </c>
       <c r="U18" s="8" t="inlineStr"/>
       <c r="V18" s="8" t="inlineStr"/>
@@ -2011,7 +2011,7 @@
       <c r="AD18" s="8" t="inlineStr"/>
       <c r="AE18" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:23</t>
+          <t>2025-10-18 11:11:22</t>
         </is>
       </c>
       <c r="AF18" s="8" t="inlineStr"/>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 43.0%</t>
+          <t>1차 매수선까지 42.9%</t>
         </is>
       </c>
       <c r="F19" s="6" t="n">
@@ -2058,26 +2058,26 @@
         <v>473720</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>474000</v>
+        <v>474500</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>43.03797468354431</v>
+        <v>42.8872497365648</v>
       </c>
       <c r="M19" s="8" t="inlineStr"/>
       <c r="N19" s="8" t="inlineStr"/>
       <c r="O19" s="6" t="n">
-        <v>427000</v>
+        <v>428000</v>
       </c>
       <c r="P19" s="7" t="n">
-        <v>58.78220140515222</v>
+        <v>58.41121495327103</v>
       </c>
       <c r="Q19" s="8" t="inlineStr"/>
       <c r="R19" s="8" t="inlineStr"/>
       <c r="S19" s="6" t="n">
-        <v>385000</v>
+        <v>386000</v>
       </c>
       <c r="T19" s="7" t="n">
-        <v>76.1038961038961</v>
+        <v>75.64766839378238</v>
       </c>
       <c r="U19" s="8" t="inlineStr"/>
       <c r="V19" s="8" t="inlineStr"/>
@@ -2091,7 +2091,7 @@
       <c r="AD19" s="8" t="inlineStr"/>
       <c r="AE19" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:24</t>
+          <t>2025-10-18 11:11:22</t>
         </is>
       </c>
       <c r="AF19" s="8" t="inlineStr"/>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 61.7%</t>
+          <t>1차 매수선까지 61.4%</t>
         </is>
       </c>
       <c r="F20" s="6" t="n">
@@ -2138,26 +2138,26 @@
         <v>25816</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>25850</v>
+        <v>25900</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>61.70212765957447</v>
+        <v>61.38996138996139</v>
       </c>
       <c r="M20" s="8" t="inlineStr"/>
       <c r="N20" s="8" t="inlineStr"/>
       <c r="O20" s="6" t="n">
-        <v>23300</v>
+        <v>23400</v>
       </c>
       <c r="P20" s="7" t="n">
-        <v>79.39914163090128</v>
+        <v>78.63247863247864</v>
       </c>
       <c r="Q20" s="8" t="inlineStr"/>
       <c r="R20" s="8" t="inlineStr"/>
       <c r="S20" s="6" t="n">
-        <v>21000</v>
+        <v>21150</v>
       </c>
       <c r="T20" s="7" t="n">
-        <v>99.04761904761905</v>
+        <v>97.63593380614657</v>
       </c>
       <c r="U20" s="8" t="inlineStr"/>
       <c r="V20" s="8" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
       <c r="AD20" s="8" t="inlineStr"/>
       <c r="AE20" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:24</t>
+          <t>2025-10-18 11:11:22</t>
         </is>
       </c>
       <c r="AF20" s="8" t="inlineStr"/>
@@ -2226,18 +2226,18 @@
       <c r="M21" s="8" t="inlineStr"/>
       <c r="N21" s="8" t="inlineStr"/>
       <c r="O21" s="6" t="n">
-        <v>110700</v>
+        <v>110800</v>
       </c>
       <c r="P21" s="7" t="n">
-        <v>73.62240289069557</v>
+        <v>73.46570397111914</v>
       </c>
       <c r="Q21" s="8" t="inlineStr"/>
       <c r="R21" s="8" t="inlineStr"/>
       <c r="S21" s="6" t="n">
-        <v>99700</v>
+        <v>99900</v>
       </c>
       <c r="T21" s="7" t="n">
-        <v>92.77833500501504</v>
+        <v>92.3923923923924</v>
       </c>
       <c r="U21" s="8" t="inlineStr"/>
       <c r="V21" s="8" t="inlineStr"/>
@@ -2251,7 +2251,7 @@
       <c r="AD21" s="8" t="inlineStr"/>
       <c r="AE21" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:24</t>
+          <t>2025-10-18 11:11:23</t>
         </is>
       </c>
       <c r="AF21" s="8" t="inlineStr"/>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 37.1%</t>
+          <t>1차 매수선까지 36.9%</t>
         </is>
       </c>
       <c r="F22" s="6" t="n">
@@ -2298,26 +2298,26 @@
         <v>54628</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>54700</v>
+        <v>54800</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>37.11151736745887</v>
+        <v>36.86131386861314</v>
       </c>
       <c r="M22" s="8" t="inlineStr"/>
       <c r="N22" s="8" t="inlineStr"/>
       <c r="O22" s="6" t="n">
-        <v>49300</v>
+        <v>49400</v>
       </c>
       <c r="P22" s="7" t="n">
-        <v>52.12981744421906</v>
+        <v>51.82186234817814</v>
       </c>
       <c r="Q22" s="8" t="inlineStr"/>
       <c r="R22" s="8" t="inlineStr"/>
       <c r="S22" s="6" t="n">
-        <v>44400</v>
+        <v>44550</v>
       </c>
       <c r="T22" s="7" t="n">
-        <v>68.91891891891892</v>
+        <v>68.35016835016835</v>
       </c>
       <c r="U22" s="8" t="inlineStr"/>
       <c r="V22" s="8" t="inlineStr"/>
@@ -2331,7 +2331,7 @@
       <c r="AD22" s="8" t="inlineStr"/>
       <c r="AE22" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:24</t>
+          <t>2025-10-18 11:11:23</t>
         </is>
       </c>
       <c r="AF22" s="8" t="inlineStr"/>
@@ -2411,7 +2411,7 @@
       <c r="AD23" s="8" t="inlineStr"/>
       <c r="AE23" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:25</t>
+          <t>2025-10-18 11:11:23</t>
         </is>
       </c>
       <c r="AF23" s="8" t="inlineStr"/>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 4.4% (접근 중!)</t>
+          <t>1차 매수선까지 4.3% (접근 중!)</t>
         </is>
       </c>
       <c r="F24" s="6" t="n">
@@ -2458,26 +2458,26 @@
         <v>8621.6</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>8630</v>
+        <v>8640</v>
       </c>
       <c r="L24" s="7" t="n">
-        <v>4.40324449594438</v>
+        <v>4.282407407407407</v>
       </c>
       <c r="M24" s="8" t="inlineStr"/>
       <c r="N24" s="8" t="inlineStr"/>
       <c r="O24" s="6" t="n">
-        <v>7780</v>
+        <v>7790</v>
       </c>
       <c r="P24" s="7" t="n">
-        <v>15.80976863753213</v>
+        <v>15.66110397946085</v>
       </c>
       <c r="Q24" s="8" t="inlineStr"/>
       <c r="R24" s="8" t="inlineStr"/>
       <c r="S24" s="6" t="n">
-        <v>7010</v>
+        <v>7030</v>
       </c>
       <c r="T24" s="7" t="n">
-        <v>28.53067047075606</v>
+        <v>28.16500711237553</v>
       </c>
       <c r="U24" s="8" t="inlineStr"/>
       <c r="V24" s="8" t="inlineStr"/>
@@ -2491,7 +2491,7 @@
       <c r="AD24" s="8" t="inlineStr"/>
       <c r="AE24" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:25</t>
+          <t>2025-10-18 11:11:24</t>
         </is>
       </c>
       <c r="AF24" s="8" t="inlineStr"/>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 19.2%</t>
+          <t>1차 매수선까지 19.1%</t>
         </is>
       </c>
       <c r="F25" s="6" t="n">
@@ -2538,26 +2538,26 @@
         <v>13321.2</v>
       </c>
       <c r="K25" s="6" t="n">
-        <v>13330</v>
+        <v>13340</v>
       </c>
       <c r="L25" s="7" t="n">
-        <v>19.20480120030007</v>
+        <v>19.11544227886057</v>
       </c>
       <c r="M25" s="8" t="inlineStr"/>
       <c r="N25" s="8" t="inlineStr"/>
       <c r="O25" s="6" t="n">
-        <v>12010</v>
+        <v>12020</v>
       </c>
       <c r="P25" s="7" t="n">
-        <v>32.30641132389675</v>
+        <v>32.1963394342762</v>
       </c>
       <c r="Q25" s="8" t="inlineStr"/>
       <c r="R25" s="8" t="inlineStr"/>
       <c r="S25" s="6" t="n">
-        <v>10820</v>
+        <v>10830</v>
       </c>
       <c r="T25" s="7" t="n">
-        <v>46.85767097966728</v>
+        <v>46.72206832871652</v>
       </c>
       <c r="U25" s="8" t="inlineStr"/>
       <c r="V25" s="8" t="inlineStr"/>
@@ -2571,7 +2571,7 @@
       <c r="AD25" s="8" t="inlineStr"/>
       <c r="AE25" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:25</t>
+          <t>2025-10-18 11:11:24</t>
         </is>
       </c>
       <c r="AF25" s="8" t="inlineStr"/>
@@ -2626,18 +2626,18 @@
       <c r="M26" s="8" t="inlineStr"/>
       <c r="N26" s="8" t="inlineStr"/>
       <c r="O26" s="6" t="n">
-        <v>44550</v>
+        <v>44600</v>
       </c>
       <c r="P26" s="7" t="n">
-        <v>29.74186307519641</v>
+        <v>29.59641255605381</v>
       </c>
       <c r="Q26" s="8" t="inlineStr"/>
       <c r="R26" s="8" t="inlineStr"/>
       <c r="S26" s="6" t="n">
-        <v>40150</v>
+        <v>40200</v>
       </c>
       <c r="T26" s="7" t="n">
-        <v>43.96014943960149</v>
+        <v>43.78109452736319</v>
       </c>
       <c r="U26" s="8" t="inlineStr"/>
       <c r="V26" s="8" t="inlineStr"/>
@@ -2651,7 +2651,7 @@
       <c r="AD26" s="8" t="inlineStr"/>
       <c r="AE26" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:26</t>
+          <t>2025-10-18 11:11:24</t>
         </is>
       </c>
       <c r="AF26" s="8" t="inlineStr"/>
@@ -2706,18 +2706,18 @@
       <c r="M27" s="8" t="inlineStr"/>
       <c r="N27" s="8" t="inlineStr"/>
       <c r="O27" s="6" t="n">
-        <v>227500</v>
+        <v>228000</v>
       </c>
       <c r="P27" s="7" t="n">
-        <v>43.2967032967033</v>
+        <v>42.98245614035088</v>
       </c>
       <c r="Q27" s="8" t="inlineStr"/>
       <c r="R27" s="8" t="inlineStr"/>
       <c r="S27" s="6" t="n">
-        <v>205500</v>
+        <v>206000</v>
       </c>
       <c r="T27" s="7" t="n">
-        <v>58.63746958637469</v>
+        <v>58.25242718446601</v>
       </c>
       <c r="U27" s="8" t="inlineStr"/>
       <c r="V27" s="8" t="inlineStr"/>
@@ -2731,7 +2731,7 @@
       <c r="AD27" s="8" t="inlineStr"/>
       <c r="AE27" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:26</t>
+          <t>2025-10-18 11:11:25</t>
         </is>
       </c>
       <c r="AF27" s="8" t="inlineStr"/>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 15.1%</t>
+          <t>1차 매수선까지 14.9%</t>
         </is>
       </c>
       <c r="F28" s="6" t="n">
@@ -2778,26 +2778,26 @@
         <v>371060</v>
       </c>
       <c r="K28" s="6" t="n">
-        <v>371500</v>
+        <v>372000</v>
       </c>
       <c r="L28" s="7" t="n">
-        <v>15.07402422611036</v>
+        <v>14.91935483870968</v>
       </c>
       <c r="M28" s="8" t="inlineStr"/>
       <c r="N28" s="8" t="inlineStr"/>
       <c r="O28" s="6" t="n">
-        <v>335000</v>
+        <v>335500</v>
       </c>
       <c r="P28" s="7" t="n">
-        <v>27.61194029850746</v>
+        <v>27.42175856929955</v>
       </c>
       <c r="Q28" s="8" t="inlineStr"/>
       <c r="R28" s="8" t="inlineStr"/>
       <c r="S28" s="6" t="n">
-        <v>302000</v>
+        <v>302500</v>
       </c>
       <c r="T28" s="7" t="n">
-        <v>41.55629139072848</v>
+        <v>41.32231404958678</v>
       </c>
       <c r="U28" s="8" t="inlineStr"/>
       <c r="V28" s="8" t="inlineStr"/>
@@ -2811,7 +2811,7 @@
       <c r="AD28" s="8" t="inlineStr"/>
       <c r="AE28" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:26</t>
+          <t>2025-10-18 11:11:25</t>
         </is>
       </c>
       <c r="AF28" s="8" t="inlineStr"/>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 25.1%</t>
+          <t>1차 매수선까지 25.0%</t>
         </is>
       </c>
       <c r="F29" s="6" t="n">
@@ -2858,26 +2858,26 @@
         <v>138716</v>
       </c>
       <c r="K29" s="6" t="n">
-        <v>138800</v>
+        <v>138900</v>
       </c>
       <c r="L29" s="7" t="n">
-        <v>25.07204610951009</v>
+        <v>24.98200143988481</v>
       </c>
       <c r="M29" s="8" t="inlineStr"/>
       <c r="N29" s="8" t="inlineStr"/>
       <c r="O29" s="6" t="n">
-        <v>125000</v>
+        <v>125200</v>
       </c>
       <c r="P29" s="7" t="n">
-        <v>38.88</v>
+        <v>38.65814696485623</v>
       </c>
       <c r="Q29" s="8" t="inlineStr"/>
       <c r="R29" s="8" t="inlineStr"/>
       <c r="S29" s="6" t="n">
-        <v>112600</v>
+        <v>112800</v>
       </c>
       <c r="T29" s="7" t="n">
-        <v>54.17406749555951</v>
+        <v>53.90070921985816</v>
       </c>
       <c r="U29" s="8" t="inlineStr"/>
       <c r="V29" s="8" t="inlineStr"/>
@@ -2891,7 +2891,7 @@
       <c r="AD29" s="8" t="inlineStr"/>
       <c r="AE29" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:26</t>
+          <t>2025-10-18 11:11:26</t>
         </is>
       </c>
       <c r="AF29" s="8" t="inlineStr"/>
@@ -2938,26 +2938,26 @@
         <v>147728</v>
       </c>
       <c r="K30" s="6" t="n">
-        <v>147800</v>
+        <v>147900</v>
       </c>
       <c r="L30" s="7" t="n">
-        <v>8.930987821380242</v>
+        <v>8.857336037863421</v>
       </c>
       <c r="M30" s="8" t="inlineStr"/>
       <c r="N30" s="8" t="inlineStr"/>
       <c r="O30" s="6" t="n">
-        <v>133100</v>
+        <v>133300</v>
       </c>
       <c r="P30" s="7" t="n">
-        <v>20.96168294515402</v>
+        <v>20.78019504876219</v>
       </c>
       <c r="Q30" s="8" t="inlineStr"/>
       <c r="R30" s="8" t="inlineStr"/>
       <c r="S30" s="6" t="n">
-        <v>119900</v>
+        <v>120100</v>
       </c>
       <c r="T30" s="7" t="n">
-        <v>34.27856547122602</v>
+        <v>34.05495420482931</v>
       </c>
       <c r="U30" s="8" t="inlineStr"/>
       <c r="V30" s="8" t="inlineStr"/>
@@ -2971,7 +2971,7 @@
       <c r="AD30" s="8" t="inlineStr"/>
       <c r="AE30" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:27</t>
+          <t>2025-10-18 11:11:26</t>
         </is>
       </c>
       <c r="AF30" s="8" t="inlineStr"/>
@@ -3018,26 +3018,26 @@
         <v>175040</v>
       </c>
       <c r="K31" s="6" t="n">
-        <v>175100</v>
+        <v>175200</v>
       </c>
       <c r="L31" s="7" t="n">
-        <v>13.93489434608795</v>
+        <v>13.86986301369863</v>
       </c>
       <c r="M31" s="8" t="inlineStr"/>
       <c r="N31" s="8" t="inlineStr"/>
       <c r="O31" s="6" t="n">
-        <v>157700</v>
+        <v>157800</v>
       </c>
       <c r="P31" s="7" t="n">
-        <v>26.50602409638554</v>
+        <v>26.42585551330798</v>
       </c>
       <c r="Q31" s="8" t="inlineStr"/>
       <c r="R31" s="8" t="inlineStr"/>
       <c r="S31" s="6" t="n">
-        <v>142000</v>
+        <v>142200</v>
       </c>
       <c r="T31" s="7" t="n">
-        <v>40.49295774647887</v>
+        <v>40.29535864978903</v>
       </c>
       <c r="U31" s="8" t="inlineStr"/>
       <c r="V31" s="8" t="inlineStr"/>
@@ -3051,7 +3051,7 @@
       <c r="AD31" s="8" t="inlineStr"/>
       <c r="AE31" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:27</t>
+          <t>2025-10-18 11:11:26</t>
         </is>
       </c>
       <c r="AF31" s="8" t="inlineStr"/>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 14.3%</t>
+          <t>1차 매수선까지 14.2%</t>
         </is>
       </c>
       <c r="F32" s="6" t="n">
@@ -3098,26 +3098,26 @@
         <v>7814.400000000001</v>
       </c>
       <c r="K32" s="6" t="n">
-        <v>7820</v>
+        <v>7830</v>
       </c>
       <c r="L32" s="7" t="n">
-        <v>14.32225063938619</v>
+        <v>14.17624521072797</v>
       </c>
       <c r="M32" s="8" t="inlineStr"/>
       <c r="N32" s="8" t="inlineStr"/>
       <c r="O32" s="6" t="n">
-        <v>7050</v>
+        <v>7060</v>
       </c>
       <c r="P32" s="7" t="n">
-        <v>26.80851063829787</v>
+        <v>26.62889518413597</v>
       </c>
       <c r="Q32" s="8" t="inlineStr"/>
       <c r="R32" s="8" t="inlineStr"/>
       <c r="S32" s="6" t="n">
-        <v>6350</v>
+        <v>6370</v>
       </c>
       <c r="T32" s="7" t="n">
-        <v>40.78740157480315</v>
+        <v>40.34536891679748</v>
       </c>
       <c r="U32" s="8" t="inlineStr"/>
       <c r="V32" s="8" t="inlineStr"/>
@@ -3131,7 +3131,7 @@
       <c r="AD32" s="8" t="inlineStr"/>
       <c r="AE32" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:27</t>
+          <t>2025-10-18 11:11:27</t>
         </is>
       </c>
       <c r="AF32" s="8" t="inlineStr"/>
@@ -3211,7 +3211,7 @@
       <c r="AD33" s="8" t="inlineStr"/>
       <c r="AE33" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:27</t>
+          <t>2025-10-18 11:11:27</t>
         </is>
       </c>
       <c r="AF33" s="8" t="inlineStr"/>
@@ -3274,10 +3274,10 @@
       <c r="Q34" s="8" t="inlineStr"/>
       <c r="R34" s="8" t="inlineStr"/>
       <c r="S34" s="6" t="n">
-        <v>31850</v>
+        <v>31900</v>
       </c>
       <c r="T34" s="7" t="n">
-        <v>102.1978021978022</v>
+        <v>101.8808777429467</v>
       </c>
       <c r="U34" s="8" t="inlineStr"/>
       <c r="V34" s="8" t="inlineStr"/>
@@ -3291,7 +3291,7 @@
       <c r="AD34" s="8" t="inlineStr"/>
       <c r="AE34" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:28</t>
+          <t>2025-10-18 11:11:27</t>
         </is>
       </c>
       <c r="AF34" s="8" t="inlineStr"/>
@@ -3354,10 +3354,10 @@
       <c r="Q35" s="8" t="inlineStr"/>
       <c r="R35" s="8" t="inlineStr"/>
       <c r="S35" s="6" t="n">
-        <v>68300</v>
+        <v>68400</v>
       </c>
       <c r="T35" s="7" t="n">
-        <v>39.67789165446559</v>
+        <v>39.47368421052632</v>
       </c>
       <c r="U35" s="8" t="inlineStr"/>
       <c r="V35" s="8" t="inlineStr"/>
@@ -3371,7 +3371,7 @@
       <c r="AD35" s="8" t="inlineStr"/>
       <c r="AE35" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:28</t>
+          <t>2025-10-18 11:11:28</t>
         </is>
       </c>
       <c r="AF35" s="8" t="inlineStr"/>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 1.2% (접근 중!)</t>
+          <t>1차 매수선까지 1.1% (접근 중!)</t>
         </is>
       </c>
       <c r="F36" s="6" t="n">
@@ -3418,26 +3418,26 @@
         <v>164336</v>
       </c>
       <c r="K36" s="6" t="n">
-        <v>164400</v>
+        <v>164500</v>
       </c>
       <c r="L36" s="7" t="n">
-        <v>1.155717761557178</v>
+        <v>1.094224924012158</v>
       </c>
       <c r="M36" s="8" t="inlineStr"/>
       <c r="N36" s="8" t="inlineStr"/>
       <c r="O36" s="6" t="n">
-        <v>148100</v>
+        <v>148200</v>
       </c>
       <c r="P36" s="7" t="n">
-        <v>12.28899392302498</v>
+        <v>12.21322537112011</v>
       </c>
       <c r="Q36" s="8" t="inlineStr"/>
       <c r="R36" s="8" t="inlineStr"/>
       <c r="S36" s="6" t="n">
-        <v>133400</v>
+        <v>133500</v>
       </c>
       <c r="T36" s="7" t="n">
-        <v>24.66266866566717</v>
+        <v>24.56928838951311</v>
       </c>
       <c r="U36" s="8" t="inlineStr"/>
       <c r="V36" s="8" t="inlineStr"/>
@@ -3451,7 +3451,7 @@
       <c r="AD36" s="8" t="inlineStr"/>
       <c r="AE36" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:28</t>
+          <t>2025-10-18 11:11:28</t>
         </is>
       </c>
       <c r="AF36" s="8" t="inlineStr"/>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 17.4%</t>
+          <t>1차 매수선까지 17.3%</t>
         </is>
       </c>
       <c r="F37" s="6" t="n">
@@ -3498,26 +3498,26 @@
         <v>361060</v>
       </c>
       <c r="K37" s="6" t="n">
-        <v>361500</v>
+        <v>362000</v>
       </c>
       <c r="L37" s="7" t="n">
-        <v>17.42738589211618</v>
+        <v>17.26519337016575</v>
       </c>
       <c r="M37" s="8" t="inlineStr"/>
       <c r="N37" s="8" t="inlineStr"/>
       <c r="O37" s="6" t="n">
-        <v>326000</v>
+        <v>326500</v>
       </c>
       <c r="P37" s="7" t="n">
-        <v>30.21472392638037</v>
+        <v>30.01531393568147</v>
       </c>
       <c r="Q37" s="8" t="inlineStr"/>
       <c r="R37" s="8" t="inlineStr"/>
       <c r="S37" s="6" t="n">
-        <v>294000</v>
+        <v>294500</v>
       </c>
       <c r="T37" s="7" t="n">
-        <v>44.38775510204081</v>
+        <v>44.14261460101868</v>
       </c>
       <c r="U37" s="8" t="inlineStr"/>
       <c r="V37" s="8" t="inlineStr"/>
@@ -3531,7 +3531,7 @@
       <c r="AD37" s="8" t="inlineStr"/>
       <c r="AE37" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:29</t>
+          <t>2025-10-18 11:11:28</t>
         </is>
       </c>
       <c r="AF37" s="8" t="inlineStr"/>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 7.7% (접근 중!)</t>
+          <t>1차 매수선까지 7.6% (접근 중!)</t>
         </is>
       </c>
       <c r="F38" s="6" t="n">
@@ -3578,26 +3578,26 @@
         <v>19864</v>
       </c>
       <c r="K38" s="6" t="n">
-        <v>19870</v>
+        <v>19880</v>
       </c>
       <c r="L38" s="7" t="n">
-        <v>7.700050327126321</v>
+        <v>7.645875251509055</v>
       </c>
       <c r="M38" s="8" t="inlineStr"/>
       <c r="N38" s="8" t="inlineStr"/>
       <c r="O38" s="6" t="n">
-        <v>17890</v>
+        <v>17910</v>
       </c>
       <c r="P38" s="7" t="n">
-        <v>19.61989938513136</v>
+        <v>19.48632049134562</v>
       </c>
       <c r="Q38" s="8" t="inlineStr"/>
       <c r="R38" s="8" t="inlineStr"/>
       <c r="S38" s="6" t="n">
-        <v>16110</v>
+        <v>16130</v>
       </c>
       <c r="T38" s="7" t="n">
-        <v>32.83674736188703</v>
+        <v>32.67203967761934</v>
       </c>
       <c r="U38" s="8" t="inlineStr"/>
       <c r="V38" s="8" t="inlineStr"/>
@@ -3611,7 +3611,7 @@
       <c r="AD38" s="8" t="inlineStr"/>
       <c r="AE38" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:29</t>
+          <t>2025-10-18 11:11:29</t>
         </is>
       </c>
       <c r="AF38" s="8" t="inlineStr"/>
@@ -3666,18 +3666,18 @@
       <c r="M39" s="8" t="inlineStr"/>
       <c r="N39" s="8" t="inlineStr"/>
       <c r="O39" s="6" t="n">
-        <v>20050</v>
+        <v>20100</v>
       </c>
       <c r="P39" s="7" t="n">
-        <v>27.93017456359102</v>
+        <v>27.61194029850746</v>
       </c>
       <c r="Q39" s="8" t="inlineStr"/>
       <c r="R39" s="8" t="inlineStr"/>
       <c r="S39" s="6" t="n">
-        <v>18050</v>
+        <v>18100</v>
       </c>
       <c r="T39" s="7" t="n">
-        <v>42.10526315789473</v>
+        <v>41.71270718232044</v>
       </c>
       <c r="U39" s="8" t="inlineStr"/>
       <c r="V39" s="8" t="inlineStr"/>
@@ -3691,7 +3691,7 @@
       <c r="AD39" s="8" t="inlineStr"/>
       <c r="AE39" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:29</t>
+          <t>2025-10-18 11:11:29</t>
         </is>
       </c>
       <c r="AF39" s="8" t="inlineStr"/>
@@ -3746,18 +3746,18 @@
       <c r="M40" s="8" t="inlineStr"/>
       <c r="N40" s="8" t="inlineStr"/>
       <c r="O40" s="6" t="n">
-        <v>15570</v>
+        <v>15580</v>
       </c>
       <c r="P40" s="7" t="n">
-        <v>29.09441233140655</v>
+        <v>29.01155327342747</v>
       </c>
       <c r="Q40" s="8" t="inlineStr"/>
       <c r="R40" s="8" t="inlineStr"/>
       <c r="S40" s="6" t="n">
-        <v>14020</v>
+        <v>14040</v>
       </c>
       <c r="T40" s="7" t="n">
-        <v>43.36661911554921</v>
+        <v>43.16239316239317</v>
       </c>
       <c r="U40" s="8" t="inlineStr"/>
       <c r="V40" s="8" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
       <c r="AD40" s="8" t="inlineStr"/>
       <c r="AE40" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:29</t>
+          <t>2025-10-18 11:11:29</t>
         </is>
       </c>
       <c r="AF40" s="8" t="inlineStr"/>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 10.2%</t>
+          <t>1차 매수선까지 10.0%</t>
         </is>
       </c>
       <c r="F41" s="6" t="n">
@@ -3818,26 +3818,26 @@
         <v>43716</v>
       </c>
       <c r="K41" s="6" t="n">
-        <v>43750</v>
+        <v>43800</v>
       </c>
       <c r="L41" s="7" t="n">
-        <v>10.17142857142857</v>
+        <v>10.04566210045662</v>
       </c>
       <c r="M41" s="8" t="inlineStr"/>
       <c r="N41" s="8" t="inlineStr"/>
       <c r="O41" s="6" t="n">
-        <v>39450</v>
+        <v>39500</v>
       </c>
       <c r="P41" s="7" t="n">
-        <v>22.17997465145754</v>
+        <v>22.0253164556962</v>
       </c>
       <c r="Q41" s="8" t="inlineStr"/>
       <c r="R41" s="8" t="inlineStr"/>
       <c r="S41" s="6" t="n">
-        <v>35550</v>
+        <v>35600</v>
       </c>
       <c r="T41" s="7" t="n">
-        <v>35.58368495077356</v>
+        <v>35.39325842696629</v>
       </c>
       <c r="U41" s="8" t="inlineStr"/>
       <c r="V41" s="8" t="inlineStr"/>
@@ -3851,7 +3851,7 @@
       <c r="AD41" s="8" t="inlineStr"/>
       <c r="AE41" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:30</t>
+          <t>2025-10-18 11:11:30</t>
         </is>
       </c>
       <c r="AF41" s="8" t="inlineStr"/>
@@ -3931,7 +3931,7 @@
       <c r="AD42" s="8" t="inlineStr"/>
       <c r="AE42" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:30</t>
+          <t>2025-10-18 11:11:30</t>
         </is>
       </c>
       <c r="AF42" s="8" t="inlineStr"/>
@@ -4011,7 +4011,7 @@
       <c r="AD43" s="8" t="inlineStr"/>
       <c r="AE43" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:30</t>
+          <t>2025-10-18 11:11:30</t>
         </is>
       </c>
       <c r="AF43" s="8" t="inlineStr"/>
@@ -4066,18 +4066,18 @@
       <c r="M44" s="8" t="inlineStr"/>
       <c r="N44" s="8" t="inlineStr"/>
       <c r="O44" s="6" t="n">
-        <v>297000</v>
+        <v>297500</v>
       </c>
       <c r="P44" s="7" t="n">
-        <v>39.22558922558922</v>
+        <v>38.99159663865547</v>
       </c>
       <c r="Q44" s="8" t="inlineStr"/>
       <c r="R44" s="8" t="inlineStr"/>
       <c r="S44" s="6" t="n">
-        <v>268000</v>
+        <v>268500</v>
       </c>
       <c r="T44" s="7" t="n">
-        <v>54.2910447761194</v>
+        <v>54.00372439478585</v>
       </c>
       <c r="U44" s="8" t="inlineStr"/>
       <c r="V44" s="8" t="inlineStr"/>
@@ -4091,7 +4091,7 @@
       <c r="AD44" s="8" t="inlineStr"/>
       <c r="AE44" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:31</t>
+          <t>2025-10-18 11:11:31</t>
         </is>
       </c>
       <c r="AF44" s="8" t="inlineStr"/>
@@ -4146,18 +4146,18 @@
       <c r="M45" s="8" t="inlineStr"/>
       <c r="N45" s="8" t="inlineStr"/>
       <c r="O45" s="6" t="n">
-        <v>143700</v>
+        <v>143800</v>
       </c>
       <c r="P45" s="7" t="n">
-        <v>38.83089770354906</v>
+        <v>38.73435326842837</v>
       </c>
       <c r="Q45" s="8" t="inlineStr"/>
       <c r="R45" s="8" t="inlineStr"/>
       <c r="S45" s="6" t="n">
-        <v>129400</v>
+        <v>129600</v>
       </c>
       <c r="T45" s="7" t="n">
-        <v>54.17310664605873</v>
+        <v>53.93518518518518</v>
       </c>
       <c r="U45" s="8" t="inlineStr"/>
       <c r="V45" s="8" t="inlineStr"/>
@@ -4171,7 +4171,7 @@
       <c r="AD45" s="8" t="inlineStr"/>
       <c r="AE45" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:31</t>
+          <t>2025-10-18 11:11:31</t>
         </is>
       </c>
       <c r="AF45" s="8" t="inlineStr"/>
@@ -4226,18 +4226,18 @@
       <c r="M46" s="8" t="inlineStr"/>
       <c r="N46" s="8" t="inlineStr"/>
       <c r="O46" s="6" t="n">
-        <v>15650</v>
+        <v>15660</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>41.85303514376997</v>
+        <v>41.7624521072797</v>
       </c>
       <c r="Q46" s="8" t="inlineStr"/>
       <c r="R46" s="8" t="inlineStr"/>
       <c r="S46" s="6" t="n">
-        <v>14090</v>
+        <v>14110</v>
       </c>
       <c r="T46" s="7" t="n">
-        <v>57.55855216465579</v>
+        <v>57.33522324592487</v>
       </c>
       <c r="U46" s="8" t="inlineStr"/>
       <c r="V46" s="8" t="inlineStr"/>
@@ -4251,7 +4251,7 @@
       <c r="AD46" s="8" t="inlineStr"/>
       <c r="AE46" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:31</t>
+          <t>2025-10-18 11:11:31</t>
         </is>
       </c>
       <c r="AF46" s="8" t="inlineStr"/>
@@ -4306,18 +4306,18 @@
       <c r="M47" s="8" t="inlineStr"/>
       <c r="N47" s="8" t="inlineStr"/>
       <c r="O47" s="6" t="n">
-        <v>1031000</v>
+        <v>1032000</v>
       </c>
       <c r="P47" s="7" t="n">
-        <v>53.24927255092143</v>
+        <v>53.10077519379846</v>
       </c>
       <c r="Q47" s="8" t="inlineStr"/>
       <c r="R47" s="8" t="inlineStr"/>
       <c r="S47" s="6" t="n">
-        <v>929000</v>
+        <v>930000</v>
       </c>
       <c r="T47" s="7" t="n">
-        <v>70.07534983853606</v>
+        <v>69.89247311827957</v>
       </c>
       <c r="U47" s="8" t="inlineStr"/>
       <c r="V47" s="8" t="inlineStr"/>
@@ -4331,7 +4331,7 @@
       <c r="AD47" s="8" t="inlineStr"/>
       <c r="AE47" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:31</t>
+          <t>2025-10-18 11:11:32</t>
         </is>
       </c>
       <c r="AF47" s="8" t="inlineStr"/>
@@ -4386,18 +4386,18 @@
       <c r="M48" s="8" t="inlineStr"/>
       <c r="N48" s="8" t="inlineStr"/>
       <c r="O48" s="6" t="n">
-        <v>355000</v>
+        <v>355500</v>
       </c>
       <c r="P48" s="7" t="n">
-        <v>21.83098591549296</v>
+        <v>21.65963431786217</v>
       </c>
       <c r="Q48" s="8" t="inlineStr"/>
       <c r="R48" s="8" t="inlineStr"/>
       <c r="S48" s="6" t="n">
-        <v>320000</v>
+        <v>320500</v>
       </c>
       <c r="T48" s="7" t="n">
-        <v>35.15625</v>
+        <v>34.94539781591264</v>
       </c>
       <c r="U48" s="8" t="inlineStr"/>
       <c r="V48" s="8" t="inlineStr"/>
@@ -4411,7 +4411,7 @@
       <c r="AD48" s="8" t="inlineStr"/>
       <c r="AE48" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:32</t>
+          <t>2025-10-18 11:11:32</t>
         </is>
       </c>
       <c r="AF48" s="8" t="inlineStr"/>
@@ -4439,7 +4439,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 20.1%</t>
+          <t>1차 매수선까지 19.9%</t>
         </is>
       </c>
       <c r="F49" s="6" t="n">
@@ -4458,26 +4458,26 @@
         <v>33362</v>
       </c>
       <c r="K49" s="6" t="n">
-        <v>33400</v>
+        <v>33450</v>
       </c>
       <c r="L49" s="7" t="n">
-        <v>20.05988023952096</v>
+        <v>19.88041853512706</v>
       </c>
       <c r="M49" s="8" t="inlineStr"/>
       <c r="N49" s="8" t="inlineStr"/>
       <c r="O49" s="6" t="n">
-        <v>30100</v>
+        <v>30200</v>
       </c>
       <c r="P49" s="7" t="n">
-        <v>33.22259136212624</v>
+        <v>32.78145695364238</v>
       </c>
       <c r="Q49" s="8" t="inlineStr"/>
       <c r="R49" s="8" t="inlineStr"/>
       <c r="S49" s="6" t="n">
-        <v>27150</v>
+        <v>27250</v>
       </c>
       <c r="T49" s="7" t="n">
-        <v>47.69797421731123</v>
+        <v>47.1559633027523</v>
       </c>
       <c r="U49" s="8" t="inlineStr"/>
       <c r="V49" s="8" t="inlineStr"/>
@@ -4491,7 +4491,7 @@
       <c r="AD49" s="8" t="inlineStr"/>
       <c r="AE49" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:32</t>
+          <t>2025-10-18 11:11:32</t>
         </is>
       </c>
       <c r="AF49" s="8" t="inlineStr"/>
@@ -4554,10 +4554,10 @@
       <c r="Q50" s="8" t="inlineStr"/>
       <c r="R50" s="8" t="inlineStr"/>
       <c r="S50" s="6" t="n">
-        <v>12040</v>
+        <v>12050</v>
       </c>
       <c r="T50" s="7" t="n">
-        <v>33.05647840531562</v>
+        <v>32.9460580912863</v>
       </c>
       <c r="U50" s="8" t="inlineStr"/>
       <c r="V50" s="8" t="inlineStr"/>
@@ -4571,7 +4571,7 @@
       <c r="AD50" s="8" t="inlineStr"/>
       <c r="AE50" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:32</t>
+          <t>2025-10-18 11:11:32</t>
         </is>
       </c>
       <c r="AF50" s="8" t="inlineStr"/>
@@ -4651,7 +4651,7 @@
       <c r="AD51" s="8" t="inlineStr"/>
       <c r="AE51" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:32</t>
+          <t>2025-10-18 11:11:33</t>
         </is>
       </c>
       <c r="AF51" s="8" t="inlineStr"/>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 26.9%</t>
+          <t>1차 매수선까지 26.8%</t>
         </is>
       </c>
       <c r="F52" s="6" t="n">
@@ -4698,26 +4698,26 @@
         <v>11183.6</v>
       </c>
       <c r="K52" s="6" t="n">
-        <v>11190</v>
+        <v>11200</v>
       </c>
       <c r="L52" s="7" t="n">
-        <v>26.89901697944593</v>
+        <v>26.78571428571428</v>
       </c>
       <c r="M52" s="8" t="inlineStr"/>
       <c r="N52" s="8" t="inlineStr"/>
       <c r="O52" s="6" t="n">
-        <v>10080</v>
+        <v>10090</v>
       </c>
       <c r="P52" s="7" t="n">
-        <v>40.87301587301587</v>
+        <v>40.73339940535183</v>
       </c>
       <c r="Q52" s="8" t="inlineStr"/>
       <c r="R52" s="8" t="inlineStr"/>
       <c r="S52" s="6" t="n">
-        <v>9080</v>
+        <v>9100</v>
       </c>
       <c r="T52" s="7" t="n">
-        <v>56.38766519823789</v>
+        <v>56.04395604395604</v>
       </c>
       <c r="U52" s="8" t="inlineStr"/>
       <c r="V52" s="8" t="inlineStr"/>
@@ -4731,7 +4731,7 @@
       <c r="AD52" s="8" t="inlineStr"/>
       <c r="AE52" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:33</t>
+          <t>2025-10-18 11:11:33</t>
         </is>
       </c>
       <c r="AF52" s="8" t="inlineStr"/>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 19.1%</t>
+          <t>1차 매수선까지 18.9%</t>
         </is>
       </c>
       <c r="F53" s="6" t="n">
@@ -4778,26 +4778,26 @@
         <v>63720</v>
       </c>
       <c r="K53" s="6" t="n">
-        <v>63800</v>
+        <v>63900</v>
       </c>
       <c r="L53" s="7" t="n">
-        <v>19.12225705329153</v>
+        <v>18.9358372456964</v>
       </c>
       <c r="M53" s="8" t="inlineStr"/>
       <c r="N53" s="8" t="inlineStr"/>
       <c r="O53" s="6" t="n">
-        <v>57500</v>
+        <v>57700</v>
       </c>
       <c r="P53" s="7" t="n">
-        <v>32.17391304347826</v>
+        <v>31.7157712305026</v>
       </c>
       <c r="Q53" s="8" t="inlineStr"/>
       <c r="R53" s="8" t="inlineStr"/>
       <c r="S53" s="6" t="n">
-        <v>51900</v>
+        <v>52100</v>
       </c>
       <c r="T53" s="7" t="n">
-        <v>46.4354527938343</v>
+        <v>45.87332053742802</v>
       </c>
       <c r="U53" s="8" t="inlineStr"/>
       <c r="V53" s="8" t="inlineStr"/>
@@ -4811,7 +4811,7 @@
       <c r="AD53" s="8" t="inlineStr"/>
       <c r="AE53" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:33</t>
+          <t>2025-10-18 11:11:33</t>
         </is>
       </c>
       <c r="AF53" s="8" t="inlineStr"/>
@@ -4874,10 +4874,10 @@
       <c r="Q54" s="8" t="inlineStr"/>
       <c r="R54" s="8" t="inlineStr"/>
       <c r="S54" s="6" t="n">
-        <v>152700</v>
+        <v>152800</v>
       </c>
       <c r="T54" s="7" t="n">
-        <v>55.20628683693517</v>
+        <v>55.10471204188482</v>
       </c>
       <c r="U54" s="8" t="inlineStr"/>
       <c r="V54" s="8" t="inlineStr"/>
@@ -4891,7 +4891,7 @@
       <c r="AD54" s="8" t="inlineStr"/>
       <c r="AE54" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:33</t>
+          <t>2025-10-18 11:11:34</t>
         </is>
       </c>
       <c r="AF54" s="8" t="inlineStr"/>
@@ -4946,18 +4946,18 @@
       <c r="M55" s="8" t="inlineStr"/>
       <c r="N55" s="8" t="inlineStr"/>
       <c r="O55" s="6" t="n">
-        <v>76200</v>
+        <v>76300</v>
       </c>
       <c r="P55" s="7" t="n">
-        <v>32.15223097112861</v>
+        <v>31.97903014416776</v>
       </c>
       <c r="Q55" s="8" t="inlineStr"/>
       <c r="R55" s="8" t="inlineStr"/>
       <c r="S55" s="6" t="n">
-        <v>68700</v>
+        <v>68800</v>
       </c>
       <c r="T55" s="7" t="n">
-        <v>46.57933042212518</v>
+        <v>46.36627906976744</v>
       </c>
       <c r="U55" s="8" t="inlineStr"/>
       <c r="V55" s="8" t="inlineStr"/>
@@ -4971,7 +4971,7 @@
       <c r="AD55" s="8" t="inlineStr"/>
       <c r="AE55" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:34</t>
+          <t>2025-10-18 11:11:34</t>
         </is>
       </c>
       <c r="AF55" s="8" t="inlineStr"/>
@@ -5026,18 +5026,18 @@
       <c r="M56" s="8" t="inlineStr"/>
       <c r="N56" s="8" t="inlineStr"/>
       <c r="O56" s="6" t="n">
-        <v>737000</v>
+        <v>738000</v>
       </c>
       <c r="P56" s="7" t="n">
-        <v>24.2876526458616</v>
+        <v>24.11924119241192</v>
       </c>
       <c r="Q56" s="8" t="inlineStr"/>
       <c r="R56" s="8" t="inlineStr"/>
       <c r="S56" s="6" t="n">
-        <v>664000</v>
+        <v>666000</v>
       </c>
       <c r="T56" s="7" t="n">
-        <v>37.95180722891566</v>
+        <v>37.53753753753754</v>
       </c>
       <c r="U56" s="8" t="inlineStr"/>
       <c r="V56" s="8" t="inlineStr"/>
@@ -5051,7 +5051,7 @@
       <c r="AD56" s="8" t="inlineStr"/>
       <c r="AE56" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:34</t>
+          <t>2025-10-18 11:11:34</t>
         </is>
       </c>
       <c r="AF56" s="8" t="inlineStr"/>
@@ -5131,7 +5131,7 @@
       <c r="AD57" s="8" t="inlineStr"/>
       <c r="AE57" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:34</t>
+          <t>2025-10-18 11:11:34</t>
         </is>
       </c>
       <c r="AF57" s="8" t="inlineStr"/>
@@ -5186,18 +5186,18 @@
       <c r="M58" s="8" t="inlineStr"/>
       <c r="N58" s="8" t="inlineStr"/>
       <c r="O58" s="6" t="n">
-        <v>21150</v>
+        <v>21200</v>
       </c>
       <c r="P58" s="7" t="n">
-        <v>39.00709219858156</v>
+        <v>38.67924528301887</v>
       </c>
       <c r="Q58" s="8" t="inlineStr"/>
       <c r="R58" s="8" t="inlineStr"/>
       <c r="S58" s="6" t="n">
-        <v>19050</v>
+        <v>19090</v>
       </c>
       <c r="T58" s="7" t="n">
-        <v>54.33070866141733</v>
+        <v>54.00733368255631</v>
       </c>
       <c r="U58" s="8" t="inlineStr"/>
       <c r="V58" s="8" t="inlineStr"/>
@@ -5211,7 +5211,7 @@
       <c r="AD58" s="8" t="inlineStr"/>
       <c r="AE58" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:34</t>
+          <t>2025-10-18 11:11:35</t>
         </is>
       </c>
       <c r="AF58" s="8" t="inlineStr"/>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 27.6%</t>
+          <t>1차 매수선까지 27.5%</t>
         </is>
       </c>
       <c r="F59" s="6" t="n">
@@ -5258,26 +5258,26 @@
         <v>158640</v>
       </c>
       <c r="K59" s="6" t="n">
-        <v>158700</v>
+        <v>158800</v>
       </c>
       <c r="L59" s="7" t="n">
-        <v>27.59924385633271</v>
+        <v>27.51889168765743</v>
       </c>
       <c r="M59" s="8" t="inlineStr"/>
       <c r="N59" s="8" t="inlineStr"/>
       <c r="O59" s="6" t="n">
-        <v>142900</v>
+        <v>143100</v>
       </c>
       <c r="P59" s="7" t="n">
-        <v>41.7074877536739</v>
+        <v>41.50943396226415</v>
       </c>
       <c r="Q59" s="8" t="inlineStr"/>
       <c r="R59" s="8" t="inlineStr"/>
       <c r="S59" s="6" t="n">
-        <v>128700</v>
+        <v>128900</v>
       </c>
       <c r="T59" s="7" t="n">
-        <v>57.34265734265735</v>
+        <v>57.09852598913887</v>
       </c>
       <c r="U59" s="8" t="inlineStr"/>
       <c r="V59" s="8" t="inlineStr"/>
@@ -5291,7 +5291,7 @@
       <c r="AD59" s="8" t="inlineStr"/>
       <c r="AE59" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:35</t>
+          <t>2025-10-18 11:11:35</t>
         </is>
       </c>
       <c r="AF59" s="8" t="inlineStr"/>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 13.6%</t>
+          <t>1차 매수선까지 13.5%</t>
         </is>
       </c>
       <c r="F60" s="6" t="n">
@@ -5338,26 +5338,26 @@
         <v>44768</v>
       </c>
       <c r="K60" s="6" t="n">
-        <v>44800</v>
+        <v>44850</v>
       </c>
       <c r="L60" s="7" t="n">
-        <v>13.61607142857143</v>
+        <v>13.48940914158306</v>
       </c>
       <c r="M60" s="8" t="inlineStr"/>
       <c r="N60" s="8" t="inlineStr"/>
       <c r="O60" s="6" t="n">
-        <v>40350</v>
+        <v>40450</v>
       </c>
       <c r="P60" s="7" t="n">
-        <v>26.14622057001239</v>
+        <v>25.83436341161928</v>
       </c>
       <c r="Q60" s="8" t="inlineStr"/>
       <c r="R60" s="8" t="inlineStr"/>
       <c r="S60" s="6" t="n">
-        <v>36350</v>
+        <v>36500</v>
       </c>
       <c r="T60" s="7" t="n">
-        <v>40.02751031636863</v>
+        <v>39.45205479452055</v>
       </c>
       <c r="U60" s="8" t="inlineStr"/>
       <c r="V60" s="8" t="inlineStr"/>
@@ -5371,7 +5371,7 @@
       <c r="AD60" s="8" t="inlineStr"/>
       <c r="AE60" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:35</t>
+          <t>2025-10-18 11:11:35</t>
         </is>
       </c>
       <c r="AF60" s="8" t="inlineStr"/>
@@ -5451,7 +5451,7 @@
       <c r="AD61" s="8" t="inlineStr"/>
       <c r="AE61" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:35</t>
+          <t>2025-10-18 11:11:36</t>
         </is>
       </c>
       <c r="AF61" s="8" t="inlineStr"/>
@@ -5506,18 +5506,18 @@
       <c r="M62" s="8" t="inlineStr"/>
       <c r="N62" s="8" t="inlineStr"/>
       <c r="O62" s="6" t="n">
-        <v>22000</v>
+        <v>22050</v>
       </c>
       <c r="P62" s="7" t="n">
-        <v>37.27272727272727</v>
+        <v>36.96145124716553</v>
       </c>
       <c r="Q62" s="8" t="inlineStr"/>
       <c r="R62" s="8" t="inlineStr"/>
       <c r="S62" s="6" t="n">
-        <v>19810</v>
+        <v>19860</v>
       </c>
       <c r="T62" s="7" t="n">
-        <v>52.44825845532559</v>
+        <v>52.06445115810675</v>
       </c>
       <c r="U62" s="8" t="inlineStr"/>
       <c r="V62" s="8" t="inlineStr"/>
@@ -5531,7 +5531,7 @@
       <c r="AD62" s="8" t="inlineStr"/>
       <c r="AE62" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:35</t>
+          <t>2025-10-18 11:11:36</t>
         </is>
       </c>
       <c r="AF62" s="8" t="inlineStr"/>
@@ -5611,7 +5611,7 @@
       <c r="AD63" s="8" t="inlineStr"/>
       <c r="AE63" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:36</t>
+          <t>2025-10-18 11:11:36</t>
         </is>
       </c>
       <c r="AF63" s="8" t="inlineStr"/>
@@ -5691,7 +5691,7 @@
       <c r="AD64" s="8" t="inlineStr"/>
       <c r="AE64" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:36</t>
+          <t>2025-10-18 11:11:36</t>
         </is>
       </c>
       <c r="AF64" s="8" t="inlineStr"/>
@@ -5754,10 +5754,10 @@
       <c r="Q65" s="8" t="inlineStr"/>
       <c r="R65" s="8" t="inlineStr"/>
       <c r="S65" s="6" t="n">
-        <v>95900</v>
+        <v>96000</v>
       </c>
       <c r="T65" s="7" t="n">
-        <v>35.97497393117831</v>
+        <v>35.83333333333334</v>
       </c>
       <c r="U65" s="8" t="inlineStr"/>
       <c r="V65" s="8" t="inlineStr"/>
@@ -5771,7 +5771,7 @@
       <c r="AD65" s="8" t="inlineStr"/>
       <c r="AE65" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:36</t>
+          <t>2025-10-18 11:11:37</t>
         </is>
       </c>
       <c r="AF65" s="8" t="inlineStr"/>
@@ -5851,7 +5851,7 @@
       <c r="AD66" s="8" t="inlineStr"/>
       <c r="AE66" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:37</t>
+          <t>2025-10-18 11:11:37</t>
         </is>
       </c>
       <c r="AF66" s="8" t="inlineStr"/>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 7.6% (접근 중!)</t>
+          <t>1차 매수선까지 7.5% (접근 중!)</t>
         </is>
       </c>
       <c r="F67" s="6" t="n">
@@ -5898,26 +5898,26 @@
         <v>8892</v>
       </c>
       <c r="K67" s="6" t="n">
-        <v>8900</v>
+        <v>8910</v>
       </c>
       <c r="L67" s="7" t="n">
-        <v>7.640449438202247</v>
+        <v>7.519640852974187</v>
       </c>
       <c r="M67" s="8" t="inlineStr"/>
       <c r="N67" s="8" t="inlineStr"/>
       <c r="O67" s="6" t="n">
-        <v>8020</v>
+        <v>8030</v>
       </c>
       <c r="P67" s="7" t="n">
-        <v>19.45137157107232</v>
+        <v>19.30261519302615</v>
       </c>
       <c r="Q67" s="8" t="inlineStr"/>
       <c r="R67" s="8" t="inlineStr"/>
       <c r="S67" s="6" t="n">
-        <v>7230</v>
+        <v>7240</v>
       </c>
       <c r="T67" s="7" t="n">
-        <v>32.50345781466113</v>
+        <v>32.32044198895028</v>
       </c>
       <c r="U67" s="8" t="inlineStr"/>
       <c r="V67" s="8" t="inlineStr"/>
@@ -5931,7 +5931,7 @@
       <c r="AD67" s="8" t="inlineStr"/>
       <c r="AE67" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:37</t>
+          <t>2025-10-18 11:11:37</t>
         </is>
       </c>
       <c r="AF67" s="8" t="inlineStr"/>
@@ -5986,18 +5986,18 @@
       <c r="M68" s="8" t="inlineStr"/>
       <c r="N68" s="8" t="inlineStr"/>
       <c r="O68" s="6" t="n">
-        <v>159300</v>
+        <v>159400</v>
       </c>
       <c r="P68" s="7" t="n">
-        <v>60.70307595731325</v>
+        <v>60.60225846925973</v>
       </c>
       <c r="Q68" s="8" t="inlineStr"/>
       <c r="R68" s="8" t="inlineStr"/>
       <c r="S68" s="6" t="n">
-        <v>143500</v>
+        <v>143600</v>
       </c>
       <c r="T68" s="7" t="n">
-        <v>78.39721254355401</v>
+        <v>78.27298050139275</v>
       </c>
       <c r="U68" s="8" t="inlineStr"/>
       <c r="V68" s="8" t="inlineStr"/>
@@ -6011,7 +6011,7 @@
       <c r="AD68" s="8" t="inlineStr"/>
       <c r="AE68" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:37</t>
+          <t>2025-10-18 11:11:37</t>
         </is>
       </c>
       <c r="AF68" s="8" t="inlineStr"/>
@@ -6066,18 +6066,18 @@
       <c r="M69" s="8" t="inlineStr"/>
       <c r="N69" s="8" t="inlineStr"/>
       <c r="O69" s="6" t="n">
-        <v>202000</v>
+        <v>202500</v>
       </c>
       <c r="P69" s="7" t="n">
-        <v>43.06930693069307</v>
+        <v>42.71604938271605</v>
       </c>
       <c r="Q69" s="8" t="inlineStr"/>
       <c r="R69" s="8" t="inlineStr"/>
       <c r="S69" s="6" t="n">
-        <v>181900</v>
+        <v>182400</v>
       </c>
       <c r="T69" s="7" t="n">
-        <v>58.87850467289719</v>
+        <v>58.44298245614035</v>
       </c>
       <c r="U69" s="8" t="inlineStr"/>
       <c r="V69" s="8" t="inlineStr"/>
@@ -6091,7 +6091,7 @@
       <c r="AD69" s="8" t="inlineStr"/>
       <c r="AE69" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:37</t>
+          <t>2025-10-18 11:11:38</t>
         </is>
       </c>
       <c r="AF69" s="8" t="inlineStr"/>
@@ -6154,10 +6154,10 @@
       <c r="Q70" s="8" t="inlineStr"/>
       <c r="R70" s="8" t="inlineStr"/>
       <c r="S70" s="6" t="n">
-        <v>62100</v>
+        <v>62200</v>
       </c>
       <c r="T70" s="7" t="n">
-        <v>52.01288244766506</v>
+        <v>51.76848874598071</v>
       </c>
       <c r="U70" s="8" t="inlineStr"/>
       <c r="V70" s="8" t="inlineStr"/>
@@ -6171,7 +6171,7 @@
       <c r="AD70" s="8" t="inlineStr"/>
       <c r="AE70" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:38</t>
+          <t>2025-10-18 11:11:38</t>
         </is>
       </c>
       <c r="AF70" s="8" t="inlineStr"/>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 17.7%</t>
+          <t>1차 매수선까지 17.5%</t>
         </is>
       </c>
       <c r="F71" s="6" t="n">
@@ -6218,26 +6218,26 @@
         <v>69424</v>
       </c>
       <c r="K71" s="6" t="n">
-        <v>69500</v>
+        <v>69600</v>
       </c>
       <c r="L71" s="7" t="n">
-        <v>17.69784172661871</v>
+        <v>17.52873563218391</v>
       </c>
       <c r="M71" s="8" t="inlineStr"/>
       <c r="N71" s="8" t="inlineStr"/>
       <c r="O71" s="6" t="n">
-        <v>62700</v>
+        <v>62800</v>
       </c>
       <c r="P71" s="7" t="n">
-        <v>30.46251993620415</v>
+        <v>30.25477707006369</v>
       </c>
       <c r="Q71" s="8" t="inlineStr"/>
       <c r="R71" s="8" t="inlineStr"/>
       <c r="S71" s="6" t="n">
-        <v>56500</v>
+        <v>56700</v>
       </c>
       <c r="T71" s="7" t="n">
-        <v>44.7787610619469</v>
+        <v>44.26807760141093</v>
       </c>
       <c r="U71" s="8" t="inlineStr"/>
       <c r="V71" s="8" t="inlineStr"/>
@@ -6251,7 +6251,7 @@
       <c r="AD71" s="8" t="inlineStr"/>
       <c r="AE71" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:38</t>
+          <t>2025-10-18 11:11:38</t>
         </is>
       </c>
       <c r="AF71" s="8" t="inlineStr"/>
@@ -6306,18 +6306,18 @@
       <c r="M72" s="8" t="inlineStr"/>
       <c r="N72" s="8" t="inlineStr"/>
       <c r="O72" s="6" t="n">
-        <v>159100</v>
+        <v>159200</v>
       </c>
       <c r="P72" s="7" t="n">
-        <v>36.0779384035198</v>
+        <v>35.99246231155779</v>
       </c>
       <c r="Q72" s="8" t="inlineStr"/>
       <c r="R72" s="8" t="inlineStr"/>
       <c r="S72" s="6" t="n">
-        <v>143300</v>
+        <v>143400</v>
       </c>
       <c r="T72" s="7" t="n">
-        <v>51.08164689462665</v>
+        <v>50.976290097629</v>
       </c>
       <c r="U72" s="8" t="inlineStr"/>
       <c r="V72" s="8" t="inlineStr"/>
@@ -6331,7 +6331,7 @@
       <c r="AD72" s="8" t="inlineStr"/>
       <c r="AE72" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:38</t>
+          <t>2025-10-18 11:11:39</t>
         </is>
       </c>
       <c r="AF72" s="8" t="inlineStr"/>
@@ -6359,7 +6359,7 @@
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>1차 매수선까지 35.3%</t>
+          <t>1차 매수선까지 35.1%</t>
         </is>
       </c>
       <c r="F73" s="6" t="n">
@@ -6378,26 +6378,26 @@
         <v>84112</v>
       </c>
       <c r="K73" s="6" t="n">
-        <v>84200</v>
+        <v>84300</v>
       </c>
       <c r="L73" s="7" t="n">
-        <v>35.27315914489311</v>
+        <v>35.11269276393831</v>
       </c>
       <c r="M73" s="8" t="inlineStr"/>
       <c r="N73" s="8" t="inlineStr"/>
       <c r="O73" s="6" t="n">
-        <v>75900</v>
+        <v>76000</v>
       </c>
       <c r="P73" s="7" t="n">
-        <v>50.06587615283268</v>
+        <v>49.86842105263158</v>
       </c>
       <c r="Q73" s="8" t="inlineStr"/>
       <c r="R73" s="8" t="inlineStr"/>
       <c r="S73" s="6" t="n">
-        <v>68400</v>
+        <v>68500</v>
       </c>
       <c r="T73" s="7" t="n">
-        <v>66.52046783625731</v>
+        <v>66.27737226277372</v>
       </c>
       <c r="U73" s="8" t="inlineStr"/>
       <c r="V73" s="8" t="inlineStr"/>
@@ -6411,7 +6411,7 @@
       <c r="AD73" s="8" t="inlineStr"/>
       <c r="AE73" s="9" t="inlineStr">
         <is>
-          <t>2025-10-18 11:08:38</t>
+          <t>2025-10-18 11:11:39</t>
         </is>
       </c>
       <c r="AF73" s="8" t="inlineStr"/>

</xml_diff>